<commit_message>
Agrega función para ajustar el ancho de columnas en la hoja "C.O. 3" del archivo Excel, asegurando que se muestre todo el texto. Implementa lógica para insertar filas adicionales si hay más de 9 materiales y copia el formato de la fila de referencia a las nuevas filas. Limpia filas de datos antes de insertar nuevos valores. Actualiza el archivo de plantilla Excel.
</commit_message>
<xml_diff>
--- a/Plantilla calificados.xlsx
+++ b/Plantilla calificados.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/alex_miramontes/Downloads/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{852784F5-C93F-3C45-97E1-EB9261E80668}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5E171CBC-534F-654B-A7A9-70E09B79F3CD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="880" windowWidth="29400" windowHeight="17540" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="880" windowWidth="29400" windowHeight="17540" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="C.O." sheetId="2" r:id="rId1"/>
@@ -752,7 +752,7 @@
     <xf numFmtId="0" fontId="16" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="17" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="176">
+  <cellXfs count="180">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="6" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
@@ -969,8 +969,6 @@
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -1003,11 +1001,119 @@
     <xf numFmtId="0" fontId="5" fillId="2" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="8" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="5" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="3" fillId="2" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="3" fillId="2" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="3" fillId="2" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="5" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="5" fillId="2" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="2" fillId="2" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="2" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="2" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="2" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="0" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="2" fontId="5" fillId="2" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="5" fillId="2" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="15" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
@@ -1015,15 +1121,6 @@
     <xf numFmtId="0" fontId="15" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="5" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="5" fillId="2" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="2" fontId="5" fillId="2" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -1036,125 +1133,44 @@
     <xf numFmtId="2" fontId="5" fillId="2" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="5" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="164" fontId="4" fillId="2" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="4" fillId="2" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="0" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="2" fontId="5" fillId="2" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="5" fillId="2" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="14" fontId="3" fillId="2" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="3" fillId="2" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="3" fillId="2" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="2" fillId="2" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="14" fontId="2" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="29" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="29" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="21" fillId="4" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="166" fontId="25" fillId="0" borderId="19" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="166" fontId="20" fillId="0" borderId="19" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="23" fillId="5" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="24" fillId="6" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="166" fontId="20" fillId="0" borderId="19" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="4" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="8" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -1879,30 +1895,30 @@
       </c>
     </row>
     <row r="2" spans="2:10" ht="14">
-      <c r="B2" s="139" t="s">
+      <c r="B2" s="150" t="s">
         <v>20</v>
       </c>
-      <c r="C2" s="140"/>
-      <c r="D2" s="140"/>
-      <c r="E2" s="140"/>
-      <c r="F2" s="140"/>
-      <c r="G2" s="140"/>
-      <c r="H2" s="140"/>
-      <c r="I2" s="140"/>
-      <c r="J2" s="141"/>
+      <c r="C2" s="151"/>
+      <c r="D2" s="151"/>
+      <c r="E2" s="151"/>
+      <c r="F2" s="151"/>
+      <c r="G2" s="151"/>
+      <c r="H2" s="151"/>
+      <c r="I2" s="151"/>
+      <c r="J2" s="152"/>
     </row>
     <row r="3" spans="2:10" ht="27" customHeight="1">
-      <c r="B3" s="142" t="s">
+      <c r="B3" s="153" t="s">
         <v>21</v>
       </c>
-      <c r="C3" s="143"/>
-      <c r="D3" s="143"/>
-      <c r="E3" s="143"/>
-      <c r="F3" s="143"/>
-      <c r="G3" s="143"/>
-      <c r="H3" s="143"/>
-      <c r="I3" s="143"/>
-      <c r="J3" s="144"/>
+      <c r="C3" s="154"/>
+      <c r="D3" s="154"/>
+      <c r="E3" s="154"/>
+      <c r="F3" s="154"/>
+      <c r="G3" s="154"/>
+      <c r="H3" s="154"/>
+      <c r="I3" s="154"/>
+      <c r="J3" s="155"/>
     </row>
     <row r="4" spans="2:10" ht="8.25" customHeight="1" thickBot="1">
       <c r="B4" s="10"/>
@@ -2163,10 +2179,10 @@
       <c r="D21" s="9"/>
       <c r="E21" s="9"/>
       <c r="F21" s="44"/>
-      <c r="G21" s="135" t="s">
+      <c r="G21" s="156" t="s">
         <v>2</v>
       </c>
-      <c r="H21" s="145"/>
+      <c r="H21" s="157"/>
       <c r="I21" s="47" t="s">
         <v>6</v>
       </c>
@@ -2182,10 +2198,10 @@
       <c r="D22" s="1"/>
       <c r="E22" s="1"/>
       <c r="F22" s="41"/>
-      <c r="G22" s="146" t="s">
+      <c r="G22" s="158" t="s">
         <v>3</v>
       </c>
-      <c r="H22" s="147"/>
+      <c r="H22" s="159"/>
       <c r="I22" s="37" t="s">
         <v>25</v>
       </c>
@@ -2201,10 +2217,10 @@
       <c r="D23" s="1"/>
       <c r="E23" s="1"/>
       <c r="F23" s="41"/>
-      <c r="G23" s="146" t="s">
+      <c r="G23" s="158" t="s">
         <v>4</v>
       </c>
-      <c r="H23" s="147"/>
+      <c r="H23" s="159"/>
       <c r="I23" s="37" t="s">
         <v>7</v>
       </c>
@@ -2218,222 +2234,222 @@
       <c r="D24" s="1"/>
       <c r="E24" s="1"/>
       <c r="F24" s="41"/>
-      <c r="G24" s="126" t="s">
+      <c r="G24" s="160" t="s">
         <v>5</v>
       </c>
-      <c r="H24" s="127"/>
+      <c r="H24" s="161"/>
       <c r="I24" s="39"/>
       <c r="J24" s="40"/>
     </row>
     <row r="25" spans="2:10" ht="13" customHeight="1">
-      <c r="B25" s="132"/>
-      <c r="C25" s="133"/>
-      <c r="D25" s="133"/>
-      <c r="E25" s="133"/>
-      <c r="F25" s="134"/>
-      <c r="G25" s="135"/>
-      <c r="H25" s="136"/>
-      <c r="I25" s="116"/>
-      <c r="J25" s="117"/>
+      <c r="B25" s="163"/>
+      <c r="C25" s="164"/>
+      <c r="D25" s="164"/>
+      <c r="E25" s="164"/>
+      <c r="F25" s="165"/>
+      <c r="G25" s="156"/>
+      <c r="H25" s="166"/>
+      <c r="I25" s="114"/>
+      <c r="J25" s="115"/>
     </row>
     <row r="26" spans="2:10" ht="13.5" customHeight="1">
-      <c r="B26" s="131"/>
-      <c r="C26" s="129"/>
-      <c r="D26" s="129"/>
-      <c r="E26" s="129"/>
-      <c r="F26" s="130"/>
-      <c r="G26" s="137"/>
-      <c r="H26" s="138"/>
-      <c r="I26" s="118"/>
-      <c r="J26" s="119"/>
+      <c r="B26" s="162"/>
+      <c r="C26" s="134"/>
+      <c r="D26" s="134"/>
+      <c r="E26" s="134"/>
+      <c r="F26" s="135"/>
+      <c r="G26" s="148"/>
+      <c r="H26" s="149"/>
+      <c r="I26" s="116"/>
+      <c r="J26" s="117"/>
     </row>
     <row r="27" spans="2:10" ht="13" customHeight="1">
-      <c r="B27" s="131"/>
-      <c r="C27" s="129"/>
-      <c r="D27" s="129"/>
-      <c r="E27" s="129"/>
-      <c r="F27" s="130"/>
-      <c r="G27" s="137"/>
-      <c r="H27" s="138"/>
-      <c r="I27" s="118"/>
-      <c r="J27" s="119"/>
+      <c r="B27" s="162"/>
+      <c r="C27" s="134"/>
+      <c r="D27" s="134"/>
+      <c r="E27" s="134"/>
+      <c r="F27" s="135"/>
+      <c r="G27" s="148"/>
+      <c r="H27" s="149"/>
+      <c r="I27" s="116"/>
+      <c r="J27" s="117"/>
     </row>
     <row r="28" spans="2:10" ht="13" customHeight="1">
-      <c r="B28" s="131"/>
-      <c r="C28" s="129"/>
-      <c r="D28" s="129"/>
-      <c r="E28" s="129"/>
-      <c r="F28" s="130"/>
-      <c r="G28" s="163"/>
-      <c r="H28" s="164"/>
-      <c r="I28" s="120"/>
-      <c r="J28" s="121"/>
+      <c r="B28" s="162"/>
+      <c r="C28" s="134"/>
+      <c r="D28" s="134"/>
+      <c r="E28" s="134"/>
+      <c r="F28" s="135"/>
+      <c r="G28" s="126"/>
+      <c r="H28" s="127"/>
+      <c r="I28" s="118"/>
+      <c r="J28" s="119"/>
     </row>
     <row r="29" spans="2:10">
-      <c r="B29" s="124" t="s">
+      <c r="B29" s="128" t="s">
         <v>10</v>
       </c>
-      <c r="C29" s="128"/>
-      <c r="D29" s="129"/>
-      <c r="E29" s="129"/>
-      <c r="F29" s="130" t="s">
+      <c r="C29" s="133"/>
+      <c r="D29" s="134"/>
+      <c r="E29" s="134"/>
+      <c r="F29" s="135" t="s">
         <v>10</v>
       </c>
-      <c r="G29" s="163"/>
-      <c r="H29" s="164"/>
-      <c r="I29" s="120"/>
-      <c r="J29" s="121"/>
+      <c r="G29" s="126"/>
+      <c r="H29" s="127"/>
+      <c r="I29" s="118"/>
+      <c r="J29" s="119"/>
     </row>
     <row r="30" spans="2:10">
-      <c r="B30" s="124" t="s">
+      <c r="B30" s="128" t="s">
         <v>10</v>
       </c>
-      <c r="C30" s="128"/>
-      <c r="D30" s="129"/>
-      <c r="E30" s="129"/>
-      <c r="F30" s="130" t="s">
+      <c r="C30" s="133"/>
+      <c r="D30" s="134"/>
+      <c r="E30" s="134"/>
+      <c r="F30" s="135" t="s">
         <v>10</v>
       </c>
-      <c r="G30" s="163"/>
-      <c r="H30" s="164"/>
-      <c r="I30" s="120"/>
-      <c r="J30" s="121"/>
+      <c r="G30" s="126"/>
+      <c r="H30" s="127"/>
+      <c r="I30" s="118"/>
+      <c r="J30" s="119"/>
     </row>
     <row r="31" spans="2:10">
-      <c r="B31" s="124" t="s">
+      <c r="B31" s="128" t="s">
         <v>10</v>
       </c>
-      <c r="C31" s="128"/>
-      <c r="D31" s="129"/>
-      <c r="E31" s="129"/>
-      <c r="F31" s="130" t="s">
+      <c r="C31" s="133"/>
+      <c r="D31" s="134"/>
+      <c r="E31" s="134"/>
+      <c r="F31" s="135" t="s">
         <v>10</v>
       </c>
-      <c r="G31" s="163"/>
-      <c r="H31" s="164"/>
-      <c r="I31" s="120"/>
-      <c r="J31" s="121"/>
+      <c r="G31" s="126"/>
+      <c r="H31" s="127"/>
+      <c r="I31" s="118"/>
+      <c r="J31" s="119"/>
     </row>
     <row r="32" spans="2:10">
-      <c r="B32" s="124" t="s">
+      <c r="B32" s="128" t="s">
         <v>10</v>
       </c>
-      <c r="C32" s="128"/>
-      <c r="D32" s="129"/>
-      <c r="E32" s="129"/>
-      <c r="F32" s="130" t="s">
+      <c r="C32" s="133"/>
+      <c r="D32" s="134"/>
+      <c r="E32" s="134"/>
+      <c r="F32" s="135" t="s">
         <v>10</v>
       </c>
-      <c r="G32" s="124"/>
-      <c r="H32" s="125"/>
-      <c r="I32" s="120"/>
-      <c r="J32" s="121"/>
+      <c r="G32" s="128"/>
+      <c r="H32" s="129"/>
+      <c r="I32" s="118"/>
+      <c r="J32" s="119"/>
     </row>
     <row r="33" spans="2:10">
-      <c r="B33" s="124" t="s">
+      <c r="B33" s="128" t="s">
         <v>10</v>
       </c>
-      <c r="C33" s="128"/>
-      <c r="D33" s="129"/>
-      <c r="E33" s="129"/>
-      <c r="F33" s="130" t="s">
+      <c r="C33" s="133"/>
+      <c r="D33" s="134"/>
+      <c r="E33" s="134"/>
+      <c r="F33" s="135" t="s">
         <v>10</v>
       </c>
-      <c r="G33" s="124"/>
-      <c r="H33" s="125"/>
-      <c r="I33" s="120"/>
-      <c r="J33" s="121"/>
+      <c r="G33" s="128"/>
+      <c r="H33" s="129"/>
+      <c r="I33" s="118"/>
+      <c r="J33" s="119"/>
     </row>
     <row r="34" spans="2:10">
-      <c r="B34" s="124" t="s">
+      <c r="B34" s="128" t="s">
         <v>10</v>
       </c>
-      <c r="C34" s="128"/>
-      <c r="D34" s="129"/>
-      <c r="E34" s="129"/>
-      <c r="F34" s="130" t="s">
+      <c r="C34" s="133"/>
+      <c r="D34" s="134"/>
+      <c r="E34" s="134"/>
+      <c r="F34" s="135" t="s">
         <v>10</v>
       </c>
-      <c r="G34" s="124"/>
-      <c r="H34" s="125"/>
-      <c r="I34" s="120"/>
-      <c r="J34" s="121"/>
+      <c r="G34" s="128"/>
+      <c r="H34" s="129"/>
+      <c r="I34" s="118"/>
+      <c r="J34" s="119"/>
     </row>
     <row r="35" spans="2:10">
-      <c r="B35" s="124" t="s">
+      <c r="B35" s="128" t="s">
         <v>10</v>
       </c>
-      <c r="C35" s="128"/>
-      <c r="D35" s="129"/>
-      <c r="E35" s="129"/>
-      <c r="F35" s="130"/>
-      <c r="G35" s="124"/>
-      <c r="H35" s="125"/>
-      <c r="I35" s="120"/>
-      <c r="J35" s="121"/>
+      <c r="C35" s="133"/>
+      <c r="D35" s="134"/>
+      <c r="E35" s="134"/>
+      <c r="F35" s="135"/>
+      <c r="G35" s="128"/>
+      <c r="H35" s="129"/>
+      <c r="I35" s="118"/>
+      <c r="J35" s="119"/>
     </row>
     <row r="36" spans="2:10">
-      <c r="B36" s="124" t="s">
+      <c r="B36" s="128" t="s">
         <v>10</v>
       </c>
-      <c r="C36" s="128"/>
-      <c r="D36" s="129"/>
-      <c r="E36" s="129"/>
-      <c r="F36" s="130"/>
-      <c r="G36" s="124"/>
-      <c r="H36" s="125"/>
-      <c r="I36" s="120"/>
-      <c r="J36" s="121"/>
+      <c r="C36" s="133"/>
+      <c r="D36" s="134"/>
+      <c r="E36" s="134"/>
+      <c r="F36" s="135"/>
+      <c r="G36" s="128"/>
+      <c r="H36" s="129"/>
+      <c r="I36" s="118"/>
+      <c r="J36" s="119"/>
     </row>
     <row r="37" spans="2:10">
-      <c r="B37" s="124"/>
-      <c r="C37" s="128"/>
-      <c r="D37" s="129"/>
-      <c r="E37" s="129"/>
-      <c r="F37" s="130"/>
-      <c r="G37" s="124"/>
-      <c r="H37" s="125"/>
-      <c r="I37" s="120"/>
-      <c r="J37" s="121"/>
+      <c r="B37" s="128"/>
+      <c r="C37" s="133"/>
+      <c r="D37" s="134"/>
+      <c r="E37" s="134"/>
+      <c r="F37" s="135"/>
+      <c r="G37" s="128"/>
+      <c r="H37" s="129"/>
+      <c r="I37" s="118"/>
+      <c r="J37" s="119"/>
     </row>
     <row r="38" spans="2:10">
-      <c r="B38" s="124"/>
-      <c r="C38" s="128"/>
-      <c r="D38" s="129"/>
-      <c r="E38" s="129"/>
-      <c r="F38" s="130"/>
-      <c r="G38" s="124"/>
-      <c r="H38" s="125"/>
-      <c r="I38" s="120"/>
-      <c r="J38" s="121"/>
+      <c r="B38" s="128"/>
+      <c r="C38" s="133"/>
+      <c r="D38" s="134"/>
+      <c r="E38" s="134"/>
+      <c r="F38" s="135"/>
+      <c r="G38" s="128"/>
+      <c r="H38" s="129"/>
+      <c r="I38" s="118"/>
+      <c r="J38" s="119"/>
     </row>
     <row r="39" spans="2:10">
-      <c r="B39" s="124"/>
-      <c r="C39" s="128"/>
-      <c r="D39" s="129"/>
-      <c r="E39" s="129"/>
-      <c r="F39" s="130"/>
-      <c r="G39" s="124"/>
-      <c r="H39" s="125"/>
-      <c r="I39" s="120"/>
-      <c r="J39" s="121"/>
+      <c r="B39" s="128"/>
+      <c r="C39" s="133"/>
+      <c r="D39" s="134"/>
+      <c r="E39" s="134"/>
+      <c r="F39" s="135"/>
+      <c r="G39" s="128"/>
+      <c r="H39" s="129"/>
+      <c r="I39" s="118"/>
+      <c r="J39" s="119"/>
     </row>
     <row r="40" spans="2:10" ht="14" thickBot="1">
-      <c r="B40" s="160"/>
-      <c r="C40" s="161"/>
-      <c r="D40" s="151"/>
-      <c r="E40" s="151"/>
-      <c r="F40" s="152"/>
-      <c r="G40" s="160"/>
-      <c r="H40" s="162"/>
-      <c r="I40" s="123"/>
-      <c r="J40" s="122"/>
+      <c r="B40" s="138"/>
+      <c r="C40" s="139"/>
+      <c r="D40" s="144"/>
+      <c r="E40" s="144"/>
+      <c r="F40" s="145"/>
+      <c r="G40" s="138"/>
+      <c r="H40" s="140"/>
+      <c r="I40" s="121"/>
+      <c r="J40" s="120"/>
     </row>
     <row r="41" spans="2:10" ht="14" thickBot="1">
-      <c r="B41" s="153" t="s">
+      <c r="B41" s="146" t="s">
         <v>29</v>
       </c>
-      <c r="C41" s="154"/>
+      <c r="C41" s="147"/>
       <c r="D41" s="6" t="s">
         <v>28</v>
       </c>
@@ -2582,8 +2598,8 @@
       <c r="J52" s="12"/>
     </row>
     <row r="53" spans="2:10" ht="20.25" customHeight="1">
-      <c r="B53" s="172"/>
-      <c r="C53" s="173"/>
+      <c r="B53" s="122"/>
+      <c r="C53" s="123"/>
       <c r="D53" s="1"/>
       <c r="E53" s="83" t="str">
         <f>B6</f>
@@ -2596,8 +2612,8 @@
       <c r="J53" s="12"/>
     </row>
     <row r="54" spans="2:10" ht="13.5" customHeight="1" thickBot="1">
-      <c r="B54" s="174"/>
-      <c r="C54" s="175"/>
+      <c r="B54" s="124"/>
+      <c r="C54" s="125"/>
       <c r="D54" s="1"/>
       <c r="E54" s="25"/>
       <c r="F54" s="62"/>
@@ -2607,8 +2623,8 @@
       <c r="J54" s="12"/>
     </row>
     <row r="55" spans="2:10" ht="9.75" customHeight="1">
-      <c r="B55" s="124"/>
-      <c r="C55" s="128"/>
+      <c r="B55" s="128"/>
+      <c r="C55" s="133"/>
       <c r="D55" s="1"/>
       <c r="E55" s="1"/>
       <c r="F55" s="5"/>
@@ -2626,15 +2642,15 @@
       <c r="E56" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="F56" s="150"/>
-      <c r="G56" s="150"/>
+      <c r="F56" s="143"/>
+      <c r="G56" s="143"/>
       <c r="H56" s="56"/>
       <c r="I56" s="1"/>
       <c r="J56" s="12"/>
     </row>
     <row r="57" spans="2:10" ht="7.5" customHeight="1" thickBot="1">
-      <c r="B57" s="158"/>
-      <c r="C57" s="159"/>
+      <c r="B57" s="136"/>
+      <c r="C57" s="137"/>
       <c r="D57" s="57"/>
       <c r="E57" s="58"/>
       <c r="F57" s="59"/>
@@ -2649,13 +2665,13 @@
       </c>
       <c r="C58" s="65"/>
       <c r="D58" s="42"/>
-      <c r="E58" s="155" t="s">
+      <c r="E58" s="130" t="s">
         <v>46</v>
       </c>
-      <c r="F58" s="156"/>
-      <c r="G58" s="156"/>
-      <c r="H58" s="156"/>
-      <c r="I58" s="157"/>
+      <c r="F58" s="131"/>
+      <c r="G58" s="131"/>
+      <c r="H58" s="131"/>
+      <c r="I58" s="132"/>
       <c r="J58" s="12"/>
     </row>
     <row r="59" spans="2:10" ht="12.75" customHeight="1">
@@ -2679,11 +2695,11 @@
       <c r="J60" s="48"/>
     </row>
     <row r="61" spans="2:10" ht="14" thickBot="1">
-      <c r="B61" s="148">
+      <c r="B61" s="141">
         <f ca="1">TODAY()</f>
         <v>46092</v>
       </c>
-      <c r="C61" s="149"/>
+      <c r="C61" s="142"/>
       <c r="E61" s="66" t="s">
         <v>42</v>
       </c>
@@ -2710,12 +2726,37 @@
     </row>
   </sheetData>
   <mergeCells count="61">
-    <mergeCell ref="B53:C54"/>
-    <mergeCell ref="G28:H28"/>
-    <mergeCell ref="G29:H29"/>
-    <mergeCell ref="G30:H30"/>
-    <mergeCell ref="G31:H31"/>
-    <mergeCell ref="G32:H32"/>
+    <mergeCell ref="G26:H26"/>
+    <mergeCell ref="G27:H27"/>
+    <mergeCell ref="B2:J2"/>
+    <mergeCell ref="B3:J3"/>
+    <mergeCell ref="G21:H21"/>
+    <mergeCell ref="G22:H22"/>
+    <mergeCell ref="G23:H23"/>
+    <mergeCell ref="G24:H24"/>
+    <mergeCell ref="B27:C27"/>
+    <mergeCell ref="B26:C26"/>
+    <mergeCell ref="B25:C25"/>
+    <mergeCell ref="D25:F25"/>
+    <mergeCell ref="D26:F26"/>
+    <mergeCell ref="D27:F27"/>
+    <mergeCell ref="G25:H25"/>
+    <mergeCell ref="B61:C61"/>
+    <mergeCell ref="B35:C35"/>
+    <mergeCell ref="D35:F35"/>
+    <mergeCell ref="B32:C32"/>
+    <mergeCell ref="D32:F32"/>
+    <mergeCell ref="F56:G56"/>
+    <mergeCell ref="B38:C38"/>
+    <mergeCell ref="D38:F38"/>
+    <mergeCell ref="B39:C39"/>
+    <mergeCell ref="D39:F39"/>
+    <mergeCell ref="D40:F40"/>
+    <mergeCell ref="B36:C36"/>
+    <mergeCell ref="D36:F36"/>
+    <mergeCell ref="B41:C41"/>
+    <mergeCell ref="B55:C55"/>
+    <mergeCell ref="B37:C37"/>
     <mergeCell ref="E58:I58"/>
     <mergeCell ref="B29:C29"/>
     <mergeCell ref="D29:F29"/>
@@ -2732,45 +2773,20 @@
     <mergeCell ref="G33:H33"/>
     <mergeCell ref="G34:H34"/>
     <mergeCell ref="G35:H35"/>
-    <mergeCell ref="B61:C61"/>
-    <mergeCell ref="B35:C35"/>
-    <mergeCell ref="D35:F35"/>
-    <mergeCell ref="B32:C32"/>
-    <mergeCell ref="D32:F32"/>
-    <mergeCell ref="F56:G56"/>
-    <mergeCell ref="B38:C38"/>
-    <mergeCell ref="D38:F38"/>
-    <mergeCell ref="B39:C39"/>
-    <mergeCell ref="D39:F39"/>
-    <mergeCell ref="D40:F40"/>
-    <mergeCell ref="B36:C36"/>
-    <mergeCell ref="D36:F36"/>
-    <mergeCell ref="B41:C41"/>
-    <mergeCell ref="B55:C55"/>
-    <mergeCell ref="B37:C37"/>
-    <mergeCell ref="G26:H26"/>
-    <mergeCell ref="G27:H27"/>
-    <mergeCell ref="B2:J2"/>
-    <mergeCell ref="B3:J3"/>
-    <mergeCell ref="G21:H21"/>
-    <mergeCell ref="G22:H22"/>
-    <mergeCell ref="G23:H23"/>
+    <mergeCell ref="B53:C54"/>
+    <mergeCell ref="G28:H28"/>
+    <mergeCell ref="G29:H29"/>
+    <mergeCell ref="G30:H30"/>
+    <mergeCell ref="G31:H31"/>
+    <mergeCell ref="G32:H32"/>
     <mergeCell ref="G36:H36"/>
     <mergeCell ref="G37:H37"/>
-    <mergeCell ref="G24:H24"/>
     <mergeCell ref="B30:C30"/>
     <mergeCell ref="D30:F30"/>
     <mergeCell ref="B34:C34"/>
     <mergeCell ref="D34:F34"/>
     <mergeCell ref="B28:C28"/>
-    <mergeCell ref="B27:C27"/>
-    <mergeCell ref="B26:C26"/>
-    <mergeCell ref="B25:C25"/>
-    <mergeCell ref="D25:F25"/>
-    <mergeCell ref="D26:F26"/>
-    <mergeCell ref="D27:F27"/>
     <mergeCell ref="D28:F28"/>
-    <mergeCell ref="G25:H25"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink ref="C12" r:id="rId1" xr:uid="{00000000-0004-0000-0000-000000000000}"/>
@@ -2798,7 +2814,7 @@
     <col min="2" max="2" width="14.6640625" customWidth="1"/>
     <col min="3" max="3" width="20.83203125" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="17.33203125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="15" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="14.1640625" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="7.83203125" customWidth="1"/>
     <col min="7" max="7" width="7.5" customWidth="1"/>
     <col min="8" max="8" width="11.5" customWidth="1"/>
@@ -2811,28 +2827,28 @@
       </c>
     </row>
     <row r="2" spans="2:9" ht="14">
-      <c r="B2" s="139" t="s">
+      <c r="B2" s="150" t="s">
         <v>20</v>
       </c>
-      <c r="C2" s="140"/>
-      <c r="D2" s="140"/>
-      <c r="E2" s="140"/>
-      <c r="F2" s="140"/>
-      <c r="G2" s="140"/>
-      <c r="H2" s="140"/>
-      <c r="I2" s="141"/>
+      <c r="C2" s="151"/>
+      <c r="D2" s="151"/>
+      <c r="E2" s="151"/>
+      <c r="F2" s="151"/>
+      <c r="G2" s="151"/>
+      <c r="H2" s="151"/>
+      <c r="I2" s="152"/>
     </row>
     <row r="3" spans="2:9" ht="27" customHeight="1">
-      <c r="B3" s="142" t="s">
+      <c r="B3" s="153" t="s">
         <v>21</v>
       </c>
-      <c r="C3" s="143"/>
-      <c r="D3" s="143"/>
-      <c r="E3" s="143"/>
-      <c r="F3" s="143"/>
-      <c r="G3" s="143"/>
-      <c r="H3" s="143"/>
-      <c r="I3" s="144"/>
+      <c r="C3" s="154"/>
+      <c r="D3" s="154"/>
+      <c r="E3" s="154"/>
+      <c r="F3" s="154"/>
+      <c r="G3" s="154"/>
+      <c r="H3" s="154"/>
+      <c r="I3" s="155"/>
     </row>
     <row r="4" spans="2:9" ht="8.25" customHeight="1" thickBot="1">
       <c r="B4" s="10"/>
@@ -2849,10 +2865,10 @@
       <c r="C5" s="28"/>
       <c r="D5" s="9"/>
       <c r="E5" s="44"/>
-      <c r="F5" s="135" t="s">
+      <c r="F5" s="156" t="s">
         <v>2</v>
       </c>
-      <c r="G5" s="145"/>
+      <c r="G5" s="157"/>
       <c r="H5" s="47" t="s">
         <v>6</v>
       </c>
@@ -2867,10 +2883,10 @@
       </c>
       <c r="D6" s="1"/>
       <c r="E6" s="41"/>
-      <c r="F6" s="146" t="s">
+      <c r="F6" s="158" t="s">
         <v>3</v>
       </c>
-      <c r="G6" s="147"/>
+      <c r="G6" s="159"/>
       <c r="H6" s="37" t="s">
         <v>25</v>
       </c>
@@ -2885,10 +2901,10 @@
       </c>
       <c r="D7" s="1"/>
       <c r="E7" s="41"/>
-      <c r="F7" s="146" t="s">
+      <c r="F7" s="158" t="s">
         <v>4</v>
       </c>
-      <c r="G7" s="147"/>
+      <c r="G7" s="159"/>
       <c r="H7" s="37" t="s">
         <v>7</v>
       </c>
@@ -2909,10 +2925,10 @@
       <c r="E8" s="104" t="s">
         <v>80</v>
       </c>
-      <c r="F8" s="147" t="s">
+      <c r="F8" s="159" t="s">
         <v>5</v>
       </c>
-      <c r="G8" s="147"/>
+      <c r="G8" s="159"/>
       <c r="H8" s="87"/>
       <c r="I8" s="38"/>
     </row>
@@ -2920,19 +2936,19 @@
       <c r="B9" s="107" t="s">
         <v>41</v>
       </c>
-      <c r="C9" s="112" t="s">
+      <c r="C9" s="110" t="s">
         <v>81</v>
       </c>
       <c r="D9" s="108" t="s">
         <v>81</v>
       </c>
-      <c r="E9" s="112" t="s">
+      <c r="E9" s="110" t="s">
         <v>81</v>
       </c>
-      <c r="F9" s="111" t="s">
+      <c r="F9" s="174" t="s">
         <v>76</v>
       </c>
-      <c r="G9" s="110"/>
+      <c r="G9" s="175"/>
       <c r="H9" s="109" t="s">
         <v>77</v>
       </c>
@@ -2947,16 +2963,16 @@
       <c r="C10" s="55" t="s">
         <v>81</v>
       </c>
-      <c r="D10" s="114" t="s">
+      <c r="D10" s="112" t="s">
         <v>81</v>
       </c>
       <c r="E10" s="55" t="s">
         <v>81</v>
       </c>
-      <c r="F10" s="45" t="s">
+      <c r="F10" s="176" t="s">
         <v>76</v>
       </c>
-      <c r="G10" s="48"/>
+      <c r="G10" s="177"/>
       <c r="H10" t="s">
         <v>77</v>
       </c>
@@ -2971,16 +2987,16 @@
       <c r="C11" s="55" t="s">
         <v>81</v>
       </c>
-      <c r="D11" s="114" t="s">
+      <c r="D11" s="112" t="s">
         <v>81</v>
       </c>
       <c r="E11" s="55" t="s">
         <v>81</v>
       </c>
-      <c r="F11" s="45" t="s">
+      <c r="F11" s="176" t="s">
         <v>76</v>
       </c>
-      <c r="G11" s="48"/>
+      <c r="G11" s="177"/>
       <c r="H11" t="s">
         <v>77</v>
       </c>
@@ -2995,16 +3011,16 @@
       <c r="C12" s="55" t="s">
         <v>81</v>
       </c>
-      <c r="D12" s="114" t="s">
+      <c r="D12" s="112" t="s">
         <v>81</v>
       </c>
       <c r="E12" s="55" t="s">
         <v>81</v>
       </c>
-      <c r="F12" s="45" t="s">
+      <c r="F12" s="176" t="s">
         <v>76</v>
       </c>
-      <c r="G12" s="48"/>
+      <c r="G12" s="177"/>
       <c r="H12" t="s">
         <v>77</v>
       </c>
@@ -3019,16 +3035,16 @@
       <c r="C13" s="55" t="s">
         <v>81</v>
       </c>
-      <c r="D13" s="114" t="s">
+      <c r="D13" s="112" t="s">
         <v>81</v>
       </c>
       <c r="E13" s="55" t="s">
         <v>81</v>
       </c>
-      <c r="F13" s="45" t="s">
+      <c r="F13" s="176" t="s">
         <v>76</v>
       </c>
-      <c r="G13" s="48"/>
+      <c r="G13" s="177"/>
       <c r="H13" t="s">
         <v>77</v>
       </c>
@@ -3043,16 +3059,16 @@
       <c r="C14" s="55" t="s">
         <v>81</v>
       </c>
-      <c r="D14" s="114" t="s">
+      <c r="D14" s="112" t="s">
         <v>81</v>
       </c>
       <c r="E14" s="55" t="s">
         <v>81</v>
       </c>
-      <c r="F14" s="45" t="s">
+      <c r="F14" s="176" t="s">
         <v>76</v>
       </c>
-      <c r="G14" s="48"/>
+      <c r="G14" s="177"/>
       <c r="H14" t="s">
         <v>77</v>
       </c>
@@ -3067,16 +3083,16 @@
       <c r="C15" s="55" t="s">
         <v>81</v>
       </c>
-      <c r="D15" s="114" t="s">
+      <c r="D15" s="112" t="s">
         <v>81</v>
       </c>
       <c r="E15" s="55" t="s">
         <v>81</v>
       </c>
-      <c r="F15" s="45" t="s">
+      <c r="F15" s="176" t="s">
         <v>76</v>
       </c>
-      <c r="G15" s="48"/>
+      <c r="G15" s="177"/>
       <c r="H15" t="s">
         <v>77</v>
       </c>
@@ -3091,16 +3107,16 @@
       <c r="C16" s="55" t="s">
         <v>81</v>
       </c>
-      <c r="D16" s="114" t="s">
+      <c r="D16" s="112" t="s">
         <v>81</v>
       </c>
       <c r="E16" s="55" t="s">
         <v>81</v>
       </c>
-      <c r="F16" s="45" t="s">
+      <c r="F16" s="176" t="s">
         <v>76</v>
       </c>
-      <c r="G16" s="48"/>
+      <c r="G16" s="177"/>
       <c r="H16" t="s">
         <v>77</v>
       </c>
@@ -3115,16 +3131,16 @@
       <c r="C17" s="55" t="s">
         <v>81</v>
       </c>
-      <c r="D17" s="114" t="s">
+      <c r="D17" s="112" t="s">
         <v>81</v>
       </c>
       <c r="E17" s="55" t="s">
         <v>81</v>
       </c>
-      <c r="F17" s="45" t="s">
+      <c r="F17" s="176" t="s">
         <v>76</v>
       </c>
-      <c r="G17" s="48"/>
+      <c r="G17" s="177"/>
       <c r="H17" t="s">
         <v>77</v>
       </c>
@@ -3139,16 +3155,16 @@
       <c r="C18" s="55" t="s">
         <v>81</v>
       </c>
-      <c r="D18" s="114" t="s">
+      <c r="D18" s="112" t="s">
         <v>81</v>
       </c>
       <c r="E18" s="55" t="s">
         <v>81</v>
       </c>
-      <c r="F18" s="45" t="s">
+      <c r="F18" s="176" t="s">
         <v>76</v>
       </c>
-      <c r="G18" s="48"/>
+      <c r="G18" s="177"/>
       <c r="H18" t="s">
         <v>77</v>
       </c>
@@ -3160,19 +3176,19 @@
       <c r="B19" s="106" t="s">
         <v>41</v>
       </c>
-      <c r="C19" s="113" t="s">
+      <c r="C19" s="111" t="s">
         <v>81</v>
       </c>
-      <c r="D19" s="115" t="s">
+      <c r="D19" s="113" t="s">
         <v>81</v>
       </c>
-      <c r="E19" s="113" t="s">
+      <c r="E19" s="111" t="s">
         <v>81</v>
       </c>
-      <c r="F19" s="17" t="s">
+      <c r="F19" s="178" t="s">
         <v>76</v>
       </c>
-      <c r="G19" s="67"/>
+      <c r="G19" s="179"/>
       <c r="H19" s="68" t="s">
         <v>77</v>
       </c>
@@ -3181,7 +3197,18 @@
       </c>
     </row>
   </sheetData>
-  <mergeCells count="6">
+  <mergeCells count="17">
+    <mergeCell ref="F19:G19"/>
+    <mergeCell ref="F14:G14"/>
+    <mergeCell ref="F15:G15"/>
+    <mergeCell ref="F16:G16"/>
+    <mergeCell ref="F17:G17"/>
+    <mergeCell ref="F18:G18"/>
+    <mergeCell ref="F9:G9"/>
+    <mergeCell ref="F10:G10"/>
+    <mergeCell ref="F11:G11"/>
+    <mergeCell ref="F12:G12"/>
+    <mergeCell ref="F13:G13"/>
     <mergeCell ref="F8:G8"/>
     <mergeCell ref="B2:I2"/>
     <mergeCell ref="B3:I3"/>
@@ -3209,7 +3236,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="2:12" ht="33" customHeight="1">
-      <c r="B1" s="170" t="s">
+      <c r="B1" s="167" t="s">
         <v>84</v>
       </c>
       <c r="C1" s="168"/>
@@ -3220,7 +3247,7 @@
       <c r="H1" s="168"/>
     </row>
     <row r="2" spans="2:12" ht="25" customHeight="1">
-      <c r="B2" s="171" t="s">
+      <c r="B2" s="169" t="s">
         <v>50</v>
       </c>
       <c r="C2" s="168"/>
@@ -3233,10 +3260,10 @@
       </c>
     </row>
     <row r="3" spans="2:12" ht="45" customHeight="1">
-      <c r="B3" s="165" t="s">
+      <c r="B3" s="170" t="s">
         <v>52</v>
       </c>
-      <c r="C3" s="165"/>
+      <c r="C3" s="170"/>
       <c r="D3" s="100" t="s">
         <v>53</v>
       </c>
@@ -3254,10 +3281,10 @@
       </c>
     </row>
     <row r="4" spans="2:12" ht="45" customHeight="1">
-      <c r="B4" s="169" t="s">
+      <c r="B4" s="171" t="s">
         <v>85</v>
       </c>
-      <c r="C4" s="165"/>
+      <c r="C4" s="170"/>
       <c r="D4" s="101" t="s">
         <v>58</v>
       </c>
@@ -3276,18 +3303,18 @@
       </c>
     </row>
     <row r="6" spans="2:12" ht="25" customHeight="1">
-      <c r="B6" s="166" t="s">
+      <c r="B6" s="172" t="s">
         <v>61</v>
       </c>
-      <c r="C6" s="166"/>
-      <c r="D6" s="166"/>
-      <c r="E6" s="166"/>
-      <c r="F6" s="166"/>
-      <c r="G6" s="166"/>
-      <c r="H6" s="166"/>
+      <c r="C6" s="172"/>
+      <c r="D6" s="172"/>
+      <c r="E6" s="172"/>
+      <c r="F6" s="172"/>
+      <c r="G6" s="172"/>
+      <c r="H6" s="172"/>
     </row>
     <row r="7" spans="2:12" ht="25" customHeight="1">
-      <c r="B7" s="166" t="s">
+      <c r="B7" s="172" t="s">
         <v>62</v>
       </c>
       <c r="C7" s="168"/>
@@ -3306,11 +3333,11 @@
       </c>
     </row>
     <row r="8" spans="2:12" ht="22" customHeight="1">
-      <c r="B8" s="169" t="s">
+      <c r="B8" s="171" t="s">
         <v>86</v>
       </c>
-      <c r="C8" s="165"/>
-      <c r="D8" s="165"/>
+      <c r="C8" s="170"/>
+      <c r="D8" s="170"/>
       <c r="E8" s="100">
         <v>37.07</v>
       </c>
@@ -3326,11 +3353,11 @@
       </c>
     </row>
     <row r="9" spans="2:12" ht="22" customHeight="1">
-      <c r="B9" s="169" t="s">
+      <c r="B9" s="171" t="s">
         <v>86</v>
       </c>
-      <c r="C9" s="165"/>
-      <c r="D9" s="165"/>
+      <c r="C9" s="170"/>
+      <c r="D9" s="170"/>
       <c r="E9" s="100">
         <v>37.07</v>
       </c>
@@ -3346,11 +3373,11 @@
       </c>
     </row>
     <row r="10" spans="2:12" ht="22" customHeight="1">
-      <c r="B10" s="169" t="s">
+      <c r="B10" s="171" t="s">
         <v>86</v>
       </c>
-      <c r="C10" s="165"/>
-      <c r="D10" s="165"/>
+      <c r="C10" s="170"/>
+      <c r="D10" s="170"/>
       <c r="E10" s="100">
         <v>44.17</v>
       </c>
@@ -3369,29 +3396,29 @@
       </c>
     </row>
     <row r="13" spans="2:12" ht="22" customHeight="1">
-      <c r="E13" s="165" t="s">
+      <c r="E13" s="170" t="s">
         <v>68</v>
       </c>
-      <c r="F13" s="165"/>
-      <c r="G13" s="165"/>
+      <c r="F13" s="170"/>
+      <c r="G13" s="170"/>
       <c r="H13" s="100">
         <f>SUM(H8:H12)</f>
         <v>1020.8983999999999</v>
       </c>
     </row>
     <row r="16" spans="2:12" ht="25" customHeight="1">
-      <c r="B16" s="166" t="s">
+      <c r="B16" s="172" t="s">
         <v>69</v>
       </c>
-      <c r="C16" s="166"/>
-      <c r="D16" s="166"/>
-      <c r="E16" s="166"/>
-      <c r="F16" s="166"/>
-      <c r="G16" s="166"/>
-      <c r="H16" s="166"/>
+      <c r="C16" s="172"/>
+      <c r="D16" s="172"/>
+      <c r="E16" s="172"/>
+      <c r="F16" s="172"/>
+      <c r="G16" s="172"/>
+      <c r="H16" s="172"/>
     </row>
     <row r="17" spans="2:16" ht="25" customHeight="1">
-      <c r="B17" s="167" t="s">
+      <c r="B17" s="173" t="s">
         <v>62</v>
       </c>
       <c r="C17" s="168"/>
@@ -3410,11 +3437,11 @@
       </c>
     </row>
     <row r="18" spans="2:16" ht="22" customHeight="1">
-      <c r="B18" s="169" t="s">
+      <c r="B18" s="171" t="s">
         <v>86</v>
       </c>
-      <c r="C18" s="165"/>
-      <c r="D18" s="165"/>
+      <c r="C18" s="170"/>
+      <c r="D18" s="170"/>
       <c r="E18" s="100">
         <v>25.33</v>
       </c>
@@ -3433,11 +3460,11 @@
       </c>
     </row>
     <row r="19" spans="2:16" ht="22" customHeight="1">
-      <c r="B19" s="169" t="s">
+      <c r="B19" s="171" t="s">
         <v>86</v>
       </c>
-      <c r="C19" s="165"/>
-      <c r="D19" s="165"/>
+      <c r="C19" s="170"/>
+      <c r="D19" s="170"/>
       <c r="E19" s="100">
         <v>1.1000000000000001</v>
       </c>
@@ -3456,34 +3483,34 @@
       </c>
     </row>
     <row r="23" spans="2:16" ht="22" customHeight="1">
-      <c r="E23" s="165" t="s">
+      <c r="E23" s="170" t="s">
         <v>68</v>
       </c>
-      <c r="F23" s="165"/>
-      <c r="G23" s="165"/>
+      <c r="F23" s="170"/>
+      <c r="G23" s="170"/>
       <c r="H23" s="100">
         <f>SUM(H18:H22)</f>
         <v>47.837293199999998</v>
       </c>
     </row>
     <row r="25" spans="2:16" ht="22" customHeight="1">
-      <c r="B25" s="165" t="s">
+      <c r="B25" s="170" t="s">
         <v>71</v>
       </c>
-      <c r="C25" s="165"/>
-      <c r="D25" s="165"/>
+      <c r="C25" s="170"/>
+      <c r="D25" s="170"/>
     </row>
     <row r="26" spans="2:16" ht="22" customHeight="1">
-      <c r="B26" s="165" t="s">
+      <c r="B26" s="170" t="s">
         <v>72</v>
       </c>
-      <c r="C26" s="165"/>
-      <c r="D26" s="165"/>
+      <c r="C26" s="170"/>
+      <c r="D26" s="170"/>
     </row>
     <row r="27" spans="2:16" ht="22" customHeight="1">
-      <c r="B27" s="165"/>
-      <c r="C27" s="165"/>
-      <c r="D27" s="165"/>
+      <c r="B27" s="170"/>
+      <c r="C27" s="170"/>
+      <c r="D27" s="170"/>
       <c r="E27" s="102" t="s">
         <v>73</v>
       </c>
@@ -3500,40 +3527,30 @@
       </c>
     </row>
     <row r="28" spans="2:16" ht="22" customHeight="1">
-      <c r="B28" s="165"/>
-      <c r="C28" s="165"/>
-      <c r="D28" s="165"/>
+      <c r="B28" s="170"/>
+      <c r="C28" s="170"/>
+      <c r="D28" s="170"/>
       <c r="F28" s="102">
         <f>H4</f>
         <v>1540.3066670000001</v>
       </c>
     </row>
     <row r="29" spans="2:16" ht="22" customHeight="1">
-      <c r="B29" s="165"/>
-      <c r="C29" s="165"/>
-      <c r="D29" s="165"/>
+      <c r="B29" s="170"/>
+      <c r="C29" s="170"/>
+      <c r="D29" s="170"/>
     </row>
     <row r="31" spans="2:16" ht="22" customHeight="1">
-      <c r="C31" s="165" t="s">
+      <c r="C31" s="170" t="s">
         <v>75</v>
       </c>
-      <c r="D31" s="165"/>
-      <c r="E31" s="165"/>
-      <c r="F31" s="165"/>
-      <c r="G31" s="165"/>
+      <c r="D31" s="170"/>
+      <c r="E31" s="170"/>
+      <c r="F31" s="170"/>
+      <c r="G31" s="170"/>
     </row>
   </sheetData>
   <mergeCells count="18">
-    <mergeCell ref="B1:H1"/>
-    <mergeCell ref="B2:G2"/>
-    <mergeCell ref="B3:C3"/>
-    <mergeCell ref="B4:C4"/>
-    <mergeCell ref="B6:H6"/>
-    <mergeCell ref="B7:D7"/>
-    <mergeCell ref="B8:D8"/>
-    <mergeCell ref="B9:D9"/>
-    <mergeCell ref="B10:D10"/>
-    <mergeCell ref="E13:G13"/>
     <mergeCell ref="B25:D25"/>
     <mergeCell ref="B26:D29"/>
     <mergeCell ref="C31:G31"/>
@@ -3542,6 +3559,16 @@
     <mergeCell ref="B18:D18"/>
     <mergeCell ref="B19:D19"/>
     <mergeCell ref="E23:G23"/>
+    <mergeCell ref="B7:D7"/>
+    <mergeCell ref="B8:D8"/>
+    <mergeCell ref="B9:D9"/>
+    <mergeCell ref="B10:D10"/>
+    <mergeCell ref="E13:G13"/>
+    <mergeCell ref="B1:H1"/>
+    <mergeCell ref="B2:G2"/>
+    <mergeCell ref="B3:C3"/>
+    <mergeCell ref="B4:C4"/>
+    <mergeCell ref="B6:H6"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Agrega una nueva plantilla Word para componentes no calificados y actualiza la lógica de gestión de países de origen en la base de datos. Se incluye un script para actualizar comentarios desde un archivo Excel y se mejora la interfaz de usuario con nuevos botones para generar certificados y reportes. Se añaden nuevas variables de estilo en CSS para mejorar la presentación.
</commit_message>
<xml_diff>
--- a/Plantilla calificados.xlsx
+++ b/Plantilla calificados.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/alex_miramontes/Downloads/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5E171CBC-534F-654B-A7A9-70E09B79F3CD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2C812F33-5BC3-DC42-8B00-DA03523CFEDE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="880" windowWidth="29400" windowHeight="17540" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="63860" yWindow="660" windowWidth="34160" windowHeight="27980" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="C.O." sheetId="2" r:id="rId1"/>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="221" uniqueCount="87">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="222" uniqueCount="88">
   <si>
     <t xml:space="preserve">DESCRIPTION OF GOOD (S) </t>
   </si>
@@ -300,6 +300,9 @@
   </si>
   <si>
     <t>Component Number / Component Name</t>
+  </si>
+  <si>
+    <t>SEE ATTACHED</t>
   </si>
 </sst>
 </file>
@@ -312,7 +315,7 @@
     <numFmt numFmtId="166" formatCode="0.000"/>
     <numFmt numFmtId="167" formatCode="0.000%"/>
   </numFmts>
-  <fonts count="30">
+  <fonts count="31">
     <font>
       <sz val="10"/>
       <name val="Arial"/>
@@ -486,6 +489,12 @@
     <font>
       <sz val="8"/>
       <color indexed="8"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="12"/>
       <name val="Arial"/>
       <family val="2"/>
     </font>
@@ -752,7 +761,7 @@
     <xf numFmtId="0" fontId="16" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="17" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="180">
+  <cellXfs count="182">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="6" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
@@ -1001,29 +1010,101 @@
     <xf numFmtId="0" fontId="5" fillId="2" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="8" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="29" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="29" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="2" fontId="5" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="5" fillId="2" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="2" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="2" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="0" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="2" fontId="5" fillId="2" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="5" fillId="2" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
     </xf>
     <xf numFmtId="14" fontId="3" fillId="2" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -1032,15 +1113,6 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="14" fontId="3" fillId="2" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="5" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="5" fillId="2" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="14" fontId="2" fillId="2" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1055,122 +1127,65 @@
     <xf numFmtId="0" fontId="5" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="5" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="2" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="4" fillId="2" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="0" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="2" fontId="5" fillId="2" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="5" fillId="2" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="2" fontId="5" fillId="2" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="5" fillId="2" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="5" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="5" fillId="2" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="8" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="25" fillId="0" borderId="19" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="5" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="6" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="166" fontId="20" fillId="0" borderId="19" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="19" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="21" fillId="4" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="166" fontId="25" fillId="0" borderId="19" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="166" fontId="20" fillId="0" borderId="19" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="5" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="6" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="2" fontId="30" fillId="2" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="30" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="30" fillId="2" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="30" fillId="2" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="30" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="30" fillId="2" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -1516,6 +1531,50 @@
         </a:p>
       </xdr:txBody>
     </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>915940</xdr:colOff>
+      <xdr:row>52</xdr:row>
+      <xdr:rowOff>46182</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>180976</xdr:colOff>
+      <xdr:row>53</xdr:row>
+      <xdr:rowOff>114974</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="3" name="Picture 2">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{C5983D78-C006-244B-A4B7-AC7FB207B492}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="1016001" y="8451273"/>
+          <a:ext cx="942975" cy="322792"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
     <xdr:clientData/>
   </xdr:twoCellAnchor>
 </xdr:wsDr>
@@ -1895,30 +1954,30 @@
       </c>
     </row>
     <row r="2" spans="2:10" ht="14">
-      <c r="B2" s="150" t="s">
+      <c r="B2" s="129" t="s">
         <v>20</v>
       </c>
-      <c r="C2" s="151"/>
-      <c r="D2" s="151"/>
-      <c r="E2" s="151"/>
-      <c r="F2" s="151"/>
-      <c r="G2" s="151"/>
-      <c r="H2" s="151"/>
-      <c r="I2" s="151"/>
-      <c r="J2" s="152"/>
+      <c r="C2" s="130"/>
+      <c r="D2" s="130"/>
+      <c r="E2" s="130"/>
+      <c r="F2" s="130"/>
+      <c r="G2" s="130"/>
+      <c r="H2" s="130"/>
+      <c r="I2" s="130"/>
+      <c r="J2" s="131"/>
     </row>
     <row r="3" spans="2:10" ht="27" customHeight="1">
-      <c r="B3" s="153" t="s">
+      <c r="B3" s="132" t="s">
         <v>21</v>
       </c>
-      <c r="C3" s="154"/>
-      <c r="D3" s="154"/>
-      <c r="E3" s="154"/>
-      <c r="F3" s="154"/>
-      <c r="G3" s="154"/>
-      <c r="H3" s="154"/>
-      <c r="I3" s="154"/>
-      <c r="J3" s="155"/>
+      <c r="C3" s="133"/>
+      <c r="D3" s="133"/>
+      <c r="E3" s="133"/>
+      <c r="F3" s="133"/>
+      <c r="G3" s="133"/>
+      <c r="H3" s="133"/>
+      <c r="I3" s="133"/>
+      <c r="J3" s="134"/>
     </row>
     <row r="4" spans="2:10" ht="8.25" customHeight="1" thickBot="1">
       <c r="B4" s="10"/>
@@ -2179,10 +2238,10 @@
       <c r="D21" s="9"/>
       <c r="E21" s="9"/>
       <c r="F21" s="44"/>
-      <c r="G21" s="156" t="s">
+      <c r="G21" s="135" t="s">
         <v>2</v>
       </c>
-      <c r="H21" s="157"/>
+      <c r="H21" s="136"/>
       <c r="I21" s="47" t="s">
         <v>6</v>
       </c>
@@ -2198,10 +2257,10 @@
       <c r="D22" s="1"/>
       <c r="E22" s="1"/>
       <c r="F22" s="41"/>
-      <c r="G22" s="158" t="s">
+      <c r="G22" s="137" t="s">
         <v>3</v>
       </c>
-      <c r="H22" s="159"/>
+      <c r="H22" s="128"/>
       <c r="I22" s="37" t="s">
         <v>25</v>
       </c>
@@ -2217,10 +2276,10 @@
       <c r="D23" s="1"/>
       <c r="E23" s="1"/>
       <c r="F23" s="41"/>
-      <c r="G23" s="158" t="s">
+      <c r="G23" s="137" t="s">
         <v>4</v>
       </c>
-      <c r="H23" s="159"/>
+      <c r="H23" s="128"/>
       <c r="I23" s="37" t="s">
         <v>7</v>
       </c>
@@ -2234,222 +2293,224 @@
       <c r="D24" s="1"/>
       <c r="E24" s="1"/>
       <c r="F24" s="41"/>
-      <c r="G24" s="160" t="s">
+      <c r="G24" s="140" t="s">
         <v>5</v>
       </c>
-      <c r="H24" s="161"/>
+      <c r="H24" s="141"/>
       <c r="I24" s="39"/>
       <c r="J24" s="40"/>
     </row>
     <row r="25" spans="2:10" ht="13" customHeight="1">
-      <c r="B25" s="163"/>
-      <c r="C25" s="164"/>
-      <c r="D25" s="164"/>
-      <c r="E25" s="164"/>
-      <c r="F25" s="165"/>
-      <c r="G25" s="156"/>
-      <c r="H25" s="166"/>
+      <c r="B25" s="176" t="s">
+        <v>87</v>
+      </c>
+      <c r="C25" s="177"/>
+      <c r="D25" s="177"/>
+      <c r="E25" s="177"/>
+      <c r="F25" s="178"/>
+      <c r="G25" s="135"/>
+      <c r="H25" s="144"/>
       <c r="I25" s="114"/>
       <c r="J25" s="115"/>
     </row>
     <row r="26" spans="2:10" ht="13.5" customHeight="1">
-      <c r="B26" s="162"/>
-      <c r="C26" s="134"/>
-      <c r="D26" s="134"/>
-      <c r="E26" s="134"/>
-      <c r="F26" s="135"/>
-      <c r="G26" s="148"/>
-      <c r="H26" s="149"/>
+      <c r="B26" s="179"/>
+      <c r="C26" s="180"/>
+      <c r="D26" s="180"/>
+      <c r="E26" s="180"/>
+      <c r="F26" s="181"/>
+      <c r="G26" s="138"/>
+      <c r="H26" s="139"/>
       <c r="I26" s="116"/>
       <c r="J26" s="117"/>
     </row>
     <row r="27" spans="2:10" ht="13" customHeight="1">
-      <c r="B27" s="162"/>
-      <c r="C27" s="134"/>
-      <c r="D27" s="134"/>
-      <c r="E27" s="134"/>
-      <c r="F27" s="135"/>
-      <c r="G27" s="148"/>
-      <c r="H27" s="149"/>
+      <c r="B27" s="179"/>
+      <c r="C27" s="180"/>
+      <c r="D27" s="180"/>
+      <c r="E27" s="180"/>
+      <c r="F27" s="181"/>
+      <c r="G27" s="138"/>
+      <c r="H27" s="139"/>
       <c r="I27" s="116"/>
       <c r="J27" s="117"/>
     </row>
     <row r="28" spans="2:10" ht="13" customHeight="1">
-      <c r="B28" s="162"/>
-      <c r="C28" s="134"/>
-      <c r="D28" s="134"/>
-      <c r="E28" s="134"/>
-      <c r="F28" s="135"/>
-      <c r="G28" s="126"/>
-      <c r="H28" s="127"/>
+      <c r="B28" s="179"/>
+      <c r="C28" s="180"/>
+      <c r="D28" s="180"/>
+      <c r="E28" s="180"/>
+      <c r="F28" s="181"/>
+      <c r="G28" s="167"/>
+      <c r="H28" s="168"/>
       <c r="I28" s="118"/>
       <c r="J28" s="119"/>
     </row>
     <row r="29" spans="2:10">
-      <c r="B29" s="128" t="s">
+      <c r="B29" s="147" t="s">
         <v>10</v>
       </c>
-      <c r="C29" s="133"/>
-      <c r="D29" s="134"/>
-      <c r="E29" s="134"/>
-      <c r="F29" s="135" t="s">
+      <c r="C29" s="148"/>
+      <c r="D29" s="142"/>
+      <c r="E29" s="142"/>
+      <c r="F29" s="143" t="s">
         <v>10</v>
       </c>
-      <c r="G29" s="126"/>
-      <c r="H29" s="127"/>
+      <c r="G29" s="167"/>
+      <c r="H29" s="168"/>
       <c r="I29" s="118"/>
       <c r="J29" s="119"/>
     </row>
     <row r="30" spans="2:10">
-      <c r="B30" s="128" t="s">
+      <c r="B30" s="147" t="s">
         <v>10</v>
       </c>
-      <c r="C30" s="133"/>
-      <c r="D30" s="134"/>
-      <c r="E30" s="134"/>
-      <c r="F30" s="135" t="s">
+      <c r="C30" s="148"/>
+      <c r="D30" s="142"/>
+      <c r="E30" s="142"/>
+      <c r="F30" s="143" t="s">
         <v>10</v>
       </c>
-      <c r="G30" s="126"/>
-      <c r="H30" s="127"/>
+      <c r="G30" s="167"/>
+      <c r="H30" s="168"/>
       <c r="I30" s="118"/>
       <c r="J30" s="119"/>
     </row>
     <row r="31" spans="2:10">
-      <c r="B31" s="128" t="s">
+      <c r="B31" s="147" t="s">
         <v>10</v>
       </c>
-      <c r="C31" s="133"/>
-      <c r="D31" s="134"/>
-      <c r="E31" s="134"/>
-      <c r="F31" s="135" t="s">
+      <c r="C31" s="148"/>
+      <c r="D31" s="142"/>
+      <c r="E31" s="142"/>
+      <c r="F31" s="143" t="s">
         <v>10</v>
       </c>
-      <c r="G31" s="126"/>
-      <c r="H31" s="127"/>
+      <c r="G31" s="167"/>
+      <c r="H31" s="168"/>
       <c r="I31" s="118"/>
       <c r="J31" s="119"/>
     </row>
     <row r="32" spans="2:10">
-      <c r="B32" s="128" t="s">
+      <c r="B32" s="147" t="s">
         <v>10</v>
       </c>
-      <c r="C32" s="133"/>
-      <c r="D32" s="134"/>
-      <c r="E32" s="134"/>
-      <c r="F32" s="135" t="s">
+      <c r="C32" s="148"/>
+      <c r="D32" s="142"/>
+      <c r="E32" s="142"/>
+      <c r="F32" s="143" t="s">
         <v>10</v>
       </c>
-      <c r="G32" s="128"/>
-      <c r="H32" s="129"/>
+      <c r="G32" s="147"/>
+      <c r="H32" s="161"/>
       <c r="I32" s="118"/>
       <c r="J32" s="119"/>
     </row>
     <row r="33" spans="2:10">
-      <c r="B33" s="128" t="s">
+      <c r="B33" s="147" t="s">
         <v>10</v>
       </c>
-      <c r="C33" s="133"/>
-      <c r="D33" s="134"/>
-      <c r="E33" s="134"/>
-      <c r="F33" s="135" t="s">
+      <c r="C33" s="148"/>
+      <c r="D33" s="142"/>
+      <c r="E33" s="142"/>
+      <c r="F33" s="143" t="s">
         <v>10</v>
       </c>
-      <c r="G33" s="128"/>
-      <c r="H33" s="129"/>
+      <c r="G33" s="147"/>
+      <c r="H33" s="161"/>
       <c r="I33" s="118"/>
       <c r="J33" s="119"/>
     </row>
     <row r="34" spans="2:10">
-      <c r="B34" s="128" t="s">
+      <c r="B34" s="147" t="s">
         <v>10</v>
       </c>
-      <c r="C34" s="133"/>
-      <c r="D34" s="134"/>
-      <c r="E34" s="134"/>
-      <c r="F34" s="135" t="s">
+      <c r="C34" s="148"/>
+      <c r="D34" s="142"/>
+      <c r="E34" s="142"/>
+      <c r="F34" s="143" t="s">
         <v>10</v>
       </c>
-      <c r="G34" s="128"/>
-      <c r="H34" s="129"/>
+      <c r="G34" s="147"/>
+      <c r="H34" s="161"/>
       <c r="I34" s="118"/>
       <c r="J34" s="119"/>
     </row>
     <row r="35" spans="2:10">
-      <c r="B35" s="128" t="s">
+      <c r="B35" s="147" t="s">
         <v>10</v>
       </c>
-      <c r="C35" s="133"/>
-      <c r="D35" s="134"/>
-      <c r="E35" s="134"/>
-      <c r="F35" s="135"/>
-      <c r="G35" s="128"/>
-      <c r="H35" s="129"/>
+      <c r="C35" s="148"/>
+      <c r="D35" s="142"/>
+      <c r="E35" s="142"/>
+      <c r="F35" s="143"/>
+      <c r="G35" s="147"/>
+      <c r="H35" s="161"/>
       <c r="I35" s="118"/>
       <c r="J35" s="119"/>
     </row>
     <row r="36" spans="2:10">
-      <c r="B36" s="128" t="s">
+      <c r="B36" s="147" t="s">
         <v>10</v>
       </c>
-      <c r="C36" s="133"/>
-      <c r="D36" s="134"/>
-      <c r="E36" s="134"/>
-      <c r="F36" s="135"/>
-      <c r="G36" s="128"/>
-      <c r="H36" s="129"/>
+      <c r="C36" s="148"/>
+      <c r="D36" s="142"/>
+      <c r="E36" s="142"/>
+      <c r="F36" s="143"/>
+      <c r="G36" s="147"/>
+      <c r="H36" s="161"/>
       <c r="I36" s="118"/>
       <c r="J36" s="119"/>
     </row>
     <row r="37" spans="2:10">
-      <c r="B37" s="128"/>
-      <c r="C37" s="133"/>
-      <c r="D37" s="134"/>
-      <c r="E37" s="134"/>
-      <c r="F37" s="135"/>
-      <c r="G37" s="128"/>
-      <c r="H37" s="129"/>
+      <c r="B37" s="147"/>
+      <c r="C37" s="148"/>
+      <c r="D37" s="142"/>
+      <c r="E37" s="142"/>
+      <c r="F37" s="143"/>
+      <c r="G37" s="147"/>
+      <c r="H37" s="161"/>
       <c r="I37" s="118"/>
       <c r="J37" s="119"/>
     </row>
     <row r="38" spans="2:10">
-      <c r="B38" s="128"/>
-      <c r="C38" s="133"/>
-      <c r="D38" s="134"/>
-      <c r="E38" s="134"/>
-      <c r="F38" s="135"/>
-      <c r="G38" s="128"/>
-      <c r="H38" s="129"/>
+      <c r="B38" s="147"/>
+      <c r="C38" s="148"/>
+      <c r="D38" s="142"/>
+      <c r="E38" s="142"/>
+      <c r="F38" s="143"/>
+      <c r="G38" s="147"/>
+      <c r="H38" s="161"/>
       <c r="I38" s="118"/>
       <c r="J38" s="119"/>
     </row>
     <row r="39" spans="2:10">
-      <c r="B39" s="128"/>
-      <c r="C39" s="133"/>
-      <c r="D39" s="134"/>
-      <c r="E39" s="134"/>
-      <c r="F39" s="135"/>
-      <c r="G39" s="128"/>
-      <c r="H39" s="129"/>
+      <c r="B39" s="147"/>
+      <c r="C39" s="148"/>
+      <c r="D39" s="142"/>
+      <c r="E39" s="142"/>
+      <c r="F39" s="143"/>
+      <c r="G39" s="147"/>
+      <c r="H39" s="161"/>
       <c r="I39" s="118"/>
       <c r="J39" s="119"/>
     </row>
     <row r="40" spans="2:10" ht="14" thickBot="1">
-      <c r="B40" s="138"/>
-      <c r="C40" s="139"/>
-      <c r="D40" s="144"/>
-      <c r="E40" s="144"/>
-      <c r="F40" s="145"/>
-      <c r="G40" s="138"/>
-      <c r="H40" s="140"/>
+      <c r="B40" s="159"/>
+      <c r="C40" s="160"/>
+      <c r="D40" s="150"/>
+      <c r="E40" s="150"/>
+      <c r="F40" s="151"/>
+      <c r="G40" s="159"/>
+      <c r="H40" s="162"/>
       <c r="I40" s="121"/>
       <c r="J40" s="120"/>
     </row>
     <row r="41" spans="2:10" ht="14" thickBot="1">
-      <c r="B41" s="146" t="s">
+      <c r="B41" s="152" t="s">
         <v>29</v>
       </c>
-      <c r="C41" s="147"/>
+      <c r="C41" s="153"/>
       <c r="D41" s="6" t="s">
         <v>28</v>
       </c>
@@ -2598,8 +2659,8 @@
       <c r="J52" s="12"/>
     </row>
     <row r="53" spans="2:10" ht="20.25" customHeight="1">
-      <c r="B53" s="122"/>
-      <c r="C53" s="123"/>
+      <c r="B53" s="163"/>
+      <c r="C53" s="164"/>
       <c r="D53" s="1"/>
       <c r="E53" s="83" t="str">
         <f>B6</f>
@@ -2612,8 +2673,8 @@
       <c r="J53" s="12"/>
     </row>
     <row r="54" spans="2:10" ht="13.5" customHeight="1" thickBot="1">
-      <c r="B54" s="124"/>
-      <c r="C54" s="125"/>
+      <c r="B54" s="165"/>
+      <c r="C54" s="166"/>
       <c r="D54" s="1"/>
       <c r="E54" s="25"/>
       <c r="F54" s="62"/>
@@ -2623,8 +2684,8 @@
       <c r="J54" s="12"/>
     </row>
     <row r="55" spans="2:10" ht="9.75" customHeight="1">
-      <c r="B55" s="128"/>
-      <c r="C55" s="133"/>
+      <c r="B55" s="147"/>
+      <c r="C55" s="148"/>
       <c r="D55" s="1"/>
       <c r="E55" s="1"/>
       <c r="F55" s="5"/>
@@ -2642,15 +2703,15 @@
       <c r="E56" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="F56" s="143"/>
-      <c r="G56" s="143"/>
+      <c r="F56" s="149"/>
+      <c r="G56" s="149"/>
       <c r="H56" s="56"/>
       <c r="I56" s="1"/>
       <c r="J56" s="12"/>
     </row>
     <row r="57" spans="2:10" ht="7.5" customHeight="1" thickBot="1">
-      <c r="B57" s="136"/>
-      <c r="C57" s="137"/>
+      <c r="B57" s="157"/>
+      <c r="C57" s="158"/>
       <c r="D57" s="57"/>
       <c r="E57" s="58"/>
       <c r="F57" s="59"/>
@@ -2665,13 +2726,13 @@
       </c>
       <c r="C58" s="65"/>
       <c r="D58" s="42"/>
-      <c r="E58" s="130" t="s">
+      <c r="E58" s="154" t="s">
         <v>46</v>
       </c>
-      <c r="F58" s="131"/>
-      <c r="G58" s="131"/>
-      <c r="H58" s="131"/>
-      <c r="I58" s="132"/>
+      <c r="F58" s="155"/>
+      <c r="G58" s="155"/>
+      <c r="H58" s="155"/>
+      <c r="I58" s="156"/>
       <c r="J58" s="12"/>
     </row>
     <row r="59" spans="2:10" ht="12.75" customHeight="1">
@@ -2695,11 +2756,11 @@
       <c r="J60" s="48"/>
     </row>
     <row r="61" spans="2:10" ht="14" thickBot="1">
-      <c r="B61" s="141">
+      <c r="B61" s="145">
         <f ca="1">TODAY()</f>
         <v>46092</v>
       </c>
-      <c r="C61" s="142"/>
+      <c r="C61" s="146"/>
       <c r="E61" s="66" t="s">
         <v>42</v>
       </c>
@@ -2725,22 +2786,36 @@
       <c r="J63" s="67"/>
     </row>
   </sheetData>
-  <mergeCells count="61">
-    <mergeCell ref="G26:H26"/>
-    <mergeCell ref="G27:H27"/>
-    <mergeCell ref="B2:J2"/>
-    <mergeCell ref="B3:J3"/>
-    <mergeCell ref="G21:H21"/>
-    <mergeCell ref="G22:H22"/>
-    <mergeCell ref="G23:H23"/>
-    <mergeCell ref="G24:H24"/>
-    <mergeCell ref="B27:C27"/>
-    <mergeCell ref="B26:C26"/>
-    <mergeCell ref="B25:C25"/>
-    <mergeCell ref="D25:F25"/>
-    <mergeCell ref="D26:F26"/>
-    <mergeCell ref="D27:F27"/>
-    <mergeCell ref="G25:H25"/>
+  <mergeCells count="54">
+    <mergeCell ref="B53:C54"/>
+    <mergeCell ref="G28:H28"/>
+    <mergeCell ref="G29:H29"/>
+    <mergeCell ref="G30:H30"/>
+    <mergeCell ref="G31:H31"/>
+    <mergeCell ref="G32:H32"/>
+    <mergeCell ref="G36:H36"/>
+    <mergeCell ref="G37:H37"/>
+    <mergeCell ref="B30:C30"/>
+    <mergeCell ref="D30:F30"/>
+    <mergeCell ref="B34:C34"/>
+    <mergeCell ref="D34:F34"/>
+    <mergeCell ref="B25:F28"/>
+    <mergeCell ref="E58:I58"/>
+    <mergeCell ref="B29:C29"/>
+    <mergeCell ref="D29:F29"/>
+    <mergeCell ref="B33:C33"/>
+    <mergeCell ref="D33:F33"/>
+    <mergeCell ref="B31:C31"/>
+    <mergeCell ref="D31:F31"/>
+    <mergeCell ref="B57:C57"/>
+    <mergeCell ref="B40:C40"/>
+    <mergeCell ref="D37:F37"/>
+    <mergeCell ref="G38:H38"/>
+    <mergeCell ref="G39:H39"/>
+    <mergeCell ref="G40:H40"/>
+    <mergeCell ref="G33:H33"/>
+    <mergeCell ref="G34:H34"/>
+    <mergeCell ref="G35:H35"/>
     <mergeCell ref="B61:C61"/>
     <mergeCell ref="B35:C35"/>
     <mergeCell ref="D35:F35"/>
@@ -2757,36 +2832,15 @@
     <mergeCell ref="B41:C41"/>
     <mergeCell ref="B55:C55"/>
     <mergeCell ref="B37:C37"/>
-    <mergeCell ref="E58:I58"/>
-    <mergeCell ref="B29:C29"/>
-    <mergeCell ref="D29:F29"/>
-    <mergeCell ref="B33:C33"/>
-    <mergeCell ref="D33:F33"/>
-    <mergeCell ref="B31:C31"/>
-    <mergeCell ref="D31:F31"/>
-    <mergeCell ref="B57:C57"/>
-    <mergeCell ref="B40:C40"/>
-    <mergeCell ref="D37:F37"/>
-    <mergeCell ref="G38:H38"/>
-    <mergeCell ref="G39:H39"/>
-    <mergeCell ref="G40:H40"/>
-    <mergeCell ref="G33:H33"/>
-    <mergeCell ref="G34:H34"/>
-    <mergeCell ref="G35:H35"/>
-    <mergeCell ref="B53:C54"/>
-    <mergeCell ref="G28:H28"/>
-    <mergeCell ref="G29:H29"/>
-    <mergeCell ref="G30:H30"/>
-    <mergeCell ref="G31:H31"/>
-    <mergeCell ref="G32:H32"/>
-    <mergeCell ref="G36:H36"/>
-    <mergeCell ref="G37:H37"/>
-    <mergeCell ref="B30:C30"/>
-    <mergeCell ref="D30:F30"/>
-    <mergeCell ref="B34:C34"/>
-    <mergeCell ref="D34:F34"/>
-    <mergeCell ref="B28:C28"/>
-    <mergeCell ref="D28:F28"/>
+    <mergeCell ref="G26:H26"/>
+    <mergeCell ref="G27:H27"/>
+    <mergeCell ref="B2:J2"/>
+    <mergeCell ref="B3:J3"/>
+    <mergeCell ref="G21:H21"/>
+    <mergeCell ref="G22:H22"/>
+    <mergeCell ref="G23:H23"/>
+    <mergeCell ref="G24:H24"/>
+    <mergeCell ref="G25:H25"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink ref="C12" r:id="rId1" xr:uid="{00000000-0004-0000-0000-000000000000}"/>
@@ -2827,28 +2881,28 @@
       </c>
     </row>
     <row r="2" spans="2:9" ht="14">
-      <c r="B2" s="150" t="s">
+      <c r="B2" s="129" t="s">
         <v>20</v>
       </c>
-      <c r="C2" s="151"/>
-      <c r="D2" s="151"/>
-      <c r="E2" s="151"/>
-      <c r="F2" s="151"/>
-      <c r="G2" s="151"/>
-      <c r="H2" s="151"/>
-      <c r="I2" s="152"/>
+      <c r="C2" s="130"/>
+      <c r="D2" s="130"/>
+      <c r="E2" s="130"/>
+      <c r="F2" s="130"/>
+      <c r="G2" s="130"/>
+      <c r="H2" s="130"/>
+      <c r="I2" s="131"/>
     </row>
     <row r="3" spans="2:9" ht="27" customHeight="1">
-      <c r="B3" s="153" t="s">
+      <c r="B3" s="132" t="s">
         <v>21</v>
       </c>
-      <c r="C3" s="154"/>
-      <c r="D3" s="154"/>
-      <c r="E3" s="154"/>
-      <c r="F3" s="154"/>
-      <c r="G3" s="154"/>
-      <c r="H3" s="154"/>
-      <c r="I3" s="155"/>
+      <c r="C3" s="133"/>
+      <c r="D3" s="133"/>
+      <c r="E3" s="133"/>
+      <c r="F3" s="133"/>
+      <c r="G3" s="133"/>
+      <c r="H3" s="133"/>
+      <c r="I3" s="134"/>
     </row>
     <row r="4" spans="2:9" ht="8.25" customHeight="1" thickBot="1">
       <c r="B4" s="10"/>
@@ -2865,10 +2919,10 @@
       <c r="C5" s="28"/>
       <c r="D5" s="9"/>
       <c r="E5" s="44"/>
-      <c r="F5" s="156" t="s">
+      <c r="F5" s="135" t="s">
         <v>2</v>
       </c>
-      <c r="G5" s="157"/>
+      <c r="G5" s="136"/>
       <c r="H5" s="47" t="s">
         <v>6</v>
       </c>
@@ -2883,10 +2937,10 @@
       </c>
       <c r="D6" s="1"/>
       <c r="E6" s="41"/>
-      <c r="F6" s="158" t="s">
+      <c r="F6" s="137" t="s">
         <v>3</v>
       </c>
-      <c r="G6" s="159"/>
+      <c r="G6" s="128"/>
       <c r="H6" s="37" t="s">
         <v>25</v>
       </c>
@@ -2901,10 +2955,10 @@
       </c>
       <c r="D7" s="1"/>
       <c r="E7" s="41"/>
-      <c r="F7" s="158" t="s">
+      <c r="F7" s="137" t="s">
         <v>4</v>
       </c>
-      <c r="G7" s="159"/>
+      <c r="G7" s="128"/>
       <c r="H7" s="37" t="s">
         <v>7</v>
       </c>
@@ -2925,10 +2979,10 @@
       <c r="E8" s="104" t="s">
         <v>80</v>
       </c>
-      <c r="F8" s="159" t="s">
+      <c r="F8" s="128" t="s">
         <v>5</v>
       </c>
-      <c r="G8" s="159"/>
+      <c r="G8" s="128"/>
       <c r="H8" s="87"/>
       <c r="I8" s="38"/>
     </row>
@@ -2945,10 +2999,10 @@
       <c r="E9" s="110" t="s">
         <v>81</v>
       </c>
-      <c r="F9" s="174" t="s">
+      <c r="F9" s="126" t="s">
         <v>76</v>
       </c>
-      <c r="G9" s="175"/>
+      <c r="G9" s="127"/>
       <c r="H9" s="109" t="s">
         <v>77</v>
       </c>
@@ -2969,10 +3023,10 @@
       <c r="E10" s="55" t="s">
         <v>81</v>
       </c>
-      <c r="F10" s="176" t="s">
+      <c r="F10" s="124" t="s">
         <v>76</v>
       </c>
-      <c r="G10" s="177"/>
+      <c r="G10" s="125"/>
       <c r="H10" t="s">
         <v>77</v>
       </c>
@@ -2993,10 +3047,10 @@
       <c r="E11" s="55" t="s">
         <v>81</v>
       </c>
-      <c r="F11" s="176" t="s">
+      <c r="F11" s="124" t="s">
         <v>76</v>
       </c>
-      <c r="G11" s="177"/>
+      <c r="G11" s="125"/>
       <c r="H11" t="s">
         <v>77</v>
       </c>
@@ -3017,10 +3071,10 @@
       <c r="E12" s="55" t="s">
         <v>81</v>
       </c>
-      <c r="F12" s="176" t="s">
+      <c r="F12" s="124" t="s">
         <v>76</v>
       </c>
-      <c r="G12" s="177"/>
+      <c r="G12" s="125"/>
       <c r="H12" t="s">
         <v>77</v>
       </c>
@@ -3041,10 +3095,10 @@
       <c r="E13" s="55" t="s">
         <v>81</v>
       </c>
-      <c r="F13" s="176" t="s">
+      <c r="F13" s="124" t="s">
         <v>76</v>
       </c>
-      <c r="G13" s="177"/>
+      <c r="G13" s="125"/>
       <c r="H13" t="s">
         <v>77</v>
       </c>
@@ -3065,10 +3119,10 @@
       <c r="E14" s="55" t="s">
         <v>81</v>
       </c>
-      <c r="F14" s="176" t="s">
+      <c r="F14" s="124" t="s">
         <v>76</v>
       </c>
-      <c r="G14" s="177"/>
+      <c r="G14" s="125"/>
       <c r="H14" t="s">
         <v>77</v>
       </c>
@@ -3089,10 +3143,10 @@
       <c r="E15" s="55" t="s">
         <v>81</v>
       </c>
-      <c r="F15" s="176" t="s">
+      <c r="F15" s="124" t="s">
         <v>76</v>
       </c>
-      <c r="G15" s="177"/>
+      <c r="G15" s="125"/>
       <c r="H15" t="s">
         <v>77</v>
       </c>
@@ -3113,10 +3167,10 @@
       <c r="E16" s="55" t="s">
         <v>81</v>
       </c>
-      <c r="F16" s="176" t="s">
+      <c r="F16" s="124" t="s">
         <v>76</v>
       </c>
-      <c r="G16" s="177"/>
+      <c r="G16" s="125"/>
       <c r="H16" t="s">
         <v>77</v>
       </c>
@@ -3137,10 +3191,10 @@
       <c r="E17" s="55" t="s">
         <v>81</v>
       </c>
-      <c r="F17" s="176" t="s">
+      <c r="F17" s="124" t="s">
         <v>76</v>
       </c>
-      <c r="G17" s="177"/>
+      <c r="G17" s="125"/>
       <c r="H17" t="s">
         <v>77</v>
       </c>
@@ -3161,10 +3215,10 @@
       <c r="E18" s="55" t="s">
         <v>81</v>
       </c>
-      <c r="F18" s="176" t="s">
+      <c r="F18" s="124" t="s">
         <v>76</v>
       </c>
-      <c r="G18" s="177"/>
+      <c r="G18" s="125"/>
       <c r="H18" t="s">
         <v>77</v>
       </c>
@@ -3185,10 +3239,10 @@
       <c r="E19" s="111" t="s">
         <v>81</v>
       </c>
-      <c r="F19" s="178" t="s">
+      <c r="F19" s="122" t="s">
         <v>76</v>
       </c>
-      <c r="G19" s="179"/>
+      <c r="G19" s="123"/>
       <c r="H19" s="68" t="s">
         <v>77</v>
       </c>
@@ -3198,23 +3252,23 @@
     </row>
   </sheetData>
   <mergeCells count="17">
+    <mergeCell ref="F8:G8"/>
+    <mergeCell ref="B2:I2"/>
+    <mergeCell ref="B3:I3"/>
+    <mergeCell ref="F5:G5"/>
+    <mergeCell ref="F6:G6"/>
+    <mergeCell ref="F7:G7"/>
+    <mergeCell ref="F9:G9"/>
+    <mergeCell ref="F10:G10"/>
+    <mergeCell ref="F11:G11"/>
+    <mergeCell ref="F12:G12"/>
+    <mergeCell ref="F13:G13"/>
     <mergeCell ref="F19:G19"/>
     <mergeCell ref="F14:G14"/>
     <mergeCell ref="F15:G15"/>
     <mergeCell ref="F16:G16"/>
     <mergeCell ref="F17:G17"/>
     <mergeCell ref="F18:G18"/>
-    <mergeCell ref="F9:G9"/>
-    <mergeCell ref="F10:G10"/>
-    <mergeCell ref="F11:G11"/>
-    <mergeCell ref="F12:G12"/>
-    <mergeCell ref="F13:G13"/>
-    <mergeCell ref="F8:G8"/>
-    <mergeCell ref="B2:I2"/>
-    <mergeCell ref="B3:I3"/>
-    <mergeCell ref="F5:G5"/>
-    <mergeCell ref="F6:G6"/>
-    <mergeCell ref="F7:G7"/>
   </mergeCells>
   <pageMargins left="0.25" right="0.17" top="0.27" bottom="0.22" header="0.25" footer="0.2"/>
   <pageSetup scale="78" orientation="portrait" r:id="rId1"/>
@@ -3236,34 +3290,34 @@
   </cols>
   <sheetData>
     <row r="1" spans="2:12" ht="33" customHeight="1">
-      <c r="B1" s="167" t="s">
+      <c r="B1" s="174" t="s">
         <v>84</v>
       </c>
-      <c r="C1" s="168"/>
-      <c r="D1" s="168"/>
-      <c r="E1" s="168"/>
-      <c r="F1" s="168"/>
-      <c r="G1" s="168"/>
-      <c r="H1" s="168"/>
+      <c r="C1" s="172"/>
+      <c r="D1" s="172"/>
+      <c r="E1" s="172"/>
+      <c r="F1" s="172"/>
+      <c r="G1" s="172"/>
+      <c r="H1" s="172"/>
     </row>
     <row r="2" spans="2:12" ht="25" customHeight="1">
-      <c r="B2" s="169" t="s">
+      <c r="B2" s="175" t="s">
         <v>50</v>
       </c>
-      <c r="C2" s="168"/>
-      <c r="D2" s="168"/>
-      <c r="E2" s="168"/>
-      <c r="F2" s="168"/>
-      <c r="G2" s="168"/>
+      <c r="C2" s="172"/>
+      <c r="D2" s="172"/>
+      <c r="E2" s="172"/>
+      <c r="F2" s="172"/>
+      <c r="G2" s="172"/>
       <c r="H2" s="97" t="s">
         <v>51</v>
       </c>
     </row>
     <row r="3" spans="2:12" ht="45" customHeight="1">
-      <c r="B3" s="170" t="s">
+      <c r="B3" s="169" t="s">
         <v>52</v>
       </c>
-      <c r="C3" s="170"/>
+      <c r="C3" s="169"/>
       <c r="D3" s="100" t="s">
         <v>53</v>
       </c>
@@ -3281,10 +3335,10 @@
       </c>
     </row>
     <row r="4" spans="2:12" ht="45" customHeight="1">
-      <c r="B4" s="171" t="s">
+      <c r="B4" s="173" t="s">
         <v>85</v>
       </c>
-      <c r="C4" s="170"/>
+      <c r="C4" s="169"/>
       <c r="D4" s="101" t="s">
         <v>58</v>
       </c>
@@ -3303,22 +3357,22 @@
       </c>
     </row>
     <row r="6" spans="2:12" ht="25" customHeight="1">
-      <c r="B6" s="172" t="s">
+      <c r="B6" s="170" t="s">
         <v>61</v>
       </c>
-      <c r="C6" s="172"/>
-      <c r="D6" s="172"/>
-      <c r="E6" s="172"/>
-      <c r="F6" s="172"/>
-      <c r="G6" s="172"/>
-      <c r="H6" s="172"/>
+      <c r="C6" s="170"/>
+      <c r="D6" s="170"/>
+      <c r="E6" s="170"/>
+      <c r="F6" s="170"/>
+      <c r="G6" s="170"/>
+      <c r="H6" s="170"/>
     </row>
     <row r="7" spans="2:12" ht="25" customHeight="1">
-      <c r="B7" s="172" t="s">
+      <c r="B7" s="170" t="s">
         <v>62</v>
       </c>
-      <c r="C7" s="168"/>
-      <c r="D7" s="168"/>
+      <c r="C7" s="172"/>
+      <c r="D7" s="172"/>
       <c r="E7" s="98" t="s">
         <v>63</v>
       </c>
@@ -3333,11 +3387,11 @@
       </c>
     </row>
     <row r="8" spans="2:12" ht="22" customHeight="1">
-      <c r="B8" s="171" t="s">
+      <c r="B8" s="173" t="s">
         <v>86</v>
       </c>
-      <c r="C8" s="170"/>
-      <c r="D8" s="170"/>
+      <c r="C8" s="169"/>
+      <c r="D8" s="169"/>
       <c r="E8" s="100">
         <v>37.07</v>
       </c>
@@ -3353,11 +3407,11 @@
       </c>
     </row>
     <row r="9" spans="2:12" ht="22" customHeight="1">
-      <c r="B9" s="171" t="s">
+      <c r="B9" s="173" t="s">
         <v>86</v>
       </c>
-      <c r="C9" s="170"/>
-      <c r="D9" s="170"/>
+      <c r="C9" s="169"/>
+      <c r="D9" s="169"/>
       <c r="E9" s="100">
         <v>37.07</v>
       </c>
@@ -3373,11 +3427,11 @@
       </c>
     </row>
     <row r="10" spans="2:12" ht="22" customHeight="1">
-      <c r="B10" s="171" t="s">
+      <c r="B10" s="173" t="s">
         <v>86</v>
       </c>
-      <c r="C10" s="170"/>
-      <c r="D10" s="170"/>
+      <c r="C10" s="169"/>
+      <c r="D10" s="169"/>
       <c r="E10" s="100">
         <v>44.17</v>
       </c>
@@ -3396,33 +3450,33 @@
       </c>
     </row>
     <row r="13" spans="2:12" ht="22" customHeight="1">
-      <c r="E13" s="170" t="s">
+      <c r="E13" s="169" t="s">
         <v>68</v>
       </c>
-      <c r="F13" s="170"/>
-      <c r="G13" s="170"/>
+      <c r="F13" s="169"/>
+      <c r="G13" s="169"/>
       <c r="H13" s="100">
         <f>SUM(H8:H12)</f>
         <v>1020.8983999999999</v>
       </c>
     </row>
     <row r="16" spans="2:12" ht="25" customHeight="1">
-      <c r="B16" s="172" t="s">
+      <c r="B16" s="170" t="s">
         <v>69</v>
       </c>
-      <c r="C16" s="172"/>
-      <c r="D16" s="172"/>
-      <c r="E16" s="172"/>
-      <c r="F16" s="172"/>
-      <c r="G16" s="172"/>
-      <c r="H16" s="172"/>
+      <c r="C16" s="170"/>
+      <c r="D16" s="170"/>
+      <c r="E16" s="170"/>
+      <c r="F16" s="170"/>
+      <c r="G16" s="170"/>
+      <c r="H16" s="170"/>
     </row>
     <row r="17" spans="2:16" ht="25" customHeight="1">
-      <c r="B17" s="173" t="s">
+      <c r="B17" s="171" t="s">
         <v>62</v>
       </c>
-      <c r="C17" s="168"/>
-      <c r="D17" s="168"/>
+      <c r="C17" s="172"/>
+      <c r="D17" s="172"/>
       <c r="E17" s="99" t="s">
         <v>63</v>
       </c>
@@ -3437,11 +3491,11 @@
       </c>
     </row>
     <row r="18" spans="2:16" ht="22" customHeight="1">
-      <c r="B18" s="171" t="s">
+      <c r="B18" s="173" t="s">
         <v>86</v>
       </c>
-      <c r="C18" s="170"/>
-      <c r="D18" s="170"/>
+      <c r="C18" s="169"/>
+      <c r="D18" s="169"/>
       <c r="E18" s="100">
         <v>25.33</v>
       </c>
@@ -3460,11 +3514,11 @@
       </c>
     </row>
     <row r="19" spans="2:16" ht="22" customHeight="1">
-      <c r="B19" s="171" t="s">
+      <c r="B19" s="173" t="s">
         <v>86</v>
       </c>
-      <c r="C19" s="170"/>
-      <c r="D19" s="170"/>
+      <c r="C19" s="169"/>
+      <c r="D19" s="169"/>
       <c r="E19" s="100">
         <v>1.1000000000000001</v>
       </c>
@@ -3483,34 +3537,34 @@
       </c>
     </row>
     <row r="23" spans="2:16" ht="22" customHeight="1">
-      <c r="E23" s="170" t="s">
+      <c r="E23" s="169" t="s">
         <v>68</v>
       </c>
-      <c r="F23" s="170"/>
-      <c r="G23" s="170"/>
+      <c r="F23" s="169"/>
+      <c r="G23" s="169"/>
       <c r="H23" s="100">
         <f>SUM(H18:H22)</f>
         <v>47.837293199999998</v>
       </c>
     </row>
     <row r="25" spans="2:16" ht="22" customHeight="1">
-      <c r="B25" s="170" t="s">
+      <c r="B25" s="169" t="s">
         <v>71</v>
       </c>
-      <c r="C25" s="170"/>
-      <c r="D25" s="170"/>
+      <c r="C25" s="169"/>
+      <c r="D25" s="169"/>
     </row>
     <row r="26" spans="2:16" ht="22" customHeight="1">
-      <c r="B26" s="170" t="s">
+      <c r="B26" s="169" t="s">
         <v>72</v>
       </c>
-      <c r="C26" s="170"/>
-      <c r="D26" s="170"/>
+      <c r="C26" s="169"/>
+      <c r="D26" s="169"/>
     </row>
     <row r="27" spans="2:16" ht="22" customHeight="1">
-      <c r="B27" s="170"/>
-      <c r="C27" s="170"/>
-      <c r="D27" s="170"/>
+      <c r="B27" s="169"/>
+      <c r="C27" s="169"/>
+      <c r="D27" s="169"/>
       <c r="E27" s="102" t="s">
         <v>73</v>
       </c>
@@ -3527,30 +3581,40 @@
       </c>
     </row>
     <row r="28" spans="2:16" ht="22" customHeight="1">
-      <c r="B28" s="170"/>
-      <c r="C28" s="170"/>
-      <c r="D28" s="170"/>
+      <c r="B28" s="169"/>
+      <c r="C28" s="169"/>
+      <c r="D28" s="169"/>
       <c r="F28" s="102">
         <f>H4</f>
         <v>1540.3066670000001</v>
       </c>
     </row>
     <row r="29" spans="2:16" ht="22" customHeight="1">
-      <c r="B29" s="170"/>
-      <c r="C29" s="170"/>
-      <c r="D29" s="170"/>
+      <c r="B29" s="169"/>
+      <c r="C29" s="169"/>
+      <c r="D29" s="169"/>
     </row>
     <row r="31" spans="2:16" ht="22" customHeight="1">
-      <c r="C31" s="170" t="s">
+      <c r="C31" s="169" t="s">
         <v>75</v>
       </c>
-      <c r="D31" s="170"/>
-      <c r="E31" s="170"/>
-      <c r="F31" s="170"/>
-      <c r="G31" s="170"/>
+      <c r="D31" s="169"/>
+      <c r="E31" s="169"/>
+      <c r="F31" s="169"/>
+      <c r="G31" s="169"/>
     </row>
   </sheetData>
   <mergeCells count="18">
+    <mergeCell ref="B1:H1"/>
+    <mergeCell ref="B2:G2"/>
+    <mergeCell ref="B3:C3"/>
+    <mergeCell ref="B4:C4"/>
+    <mergeCell ref="B6:H6"/>
+    <mergeCell ref="B7:D7"/>
+    <mergeCell ref="B8:D8"/>
+    <mergeCell ref="B9:D9"/>
+    <mergeCell ref="B10:D10"/>
+    <mergeCell ref="E13:G13"/>
     <mergeCell ref="B25:D25"/>
     <mergeCell ref="B26:D29"/>
     <mergeCell ref="C31:G31"/>
@@ -3559,16 +3623,6 @@
     <mergeCell ref="B18:D18"/>
     <mergeCell ref="B19:D19"/>
     <mergeCell ref="E23:G23"/>
-    <mergeCell ref="B7:D7"/>
-    <mergeCell ref="B8:D8"/>
-    <mergeCell ref="B9:D9"/>
-    <mergeCell ref="B10:D10"/>
-    <mergeCell ref="E13:G13"/>
-    <mergeCell ref="B1:H1"/>
-    <mergeCell ref="B2:G2"/>
-    <mergeCell ref="B3:C3"/>
-    <mergeCell ref="B4:C4"/>
-    <mergeCell ref="B6:H6"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Implementa nuevas funciones en main.py para manejar la lógica de fechas en certificados y mejorar la generación de PDFs. Se actualiza la lógica de sincronización de materiales en crud.py para evitar violaciones de unicidad en la base de datos. Se añaden nuevos estilos CSS y botones en las plantillas para mejorar la interfaz de usuario y la experiencia de descarga de informes. Se ajustan las plantillas de análisis y simulación para incluir nuevas funcionalidades y mejorar la presentación de datos.
</commit_message>
<xml_diff>
--- a/Plantilla calificados.xlsx
+++ b/Plantilla calificados.xlsx
@@ -1,21 +1,20 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10308"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10315"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/alex_miramontes/Downloads/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/alex_miramontes/freepoint/Proyectos Alex /LeoniRPA/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2C812F33-5BC3-DC42-8B00-DA03523CFEDE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D4A6D448-7EA2-D740-827D-6C5F552B7F2C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="63860" yWindow="660" windowWidth="34160" windowHeight="27980" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="740" windowWidth="29400" windowHeight="18380" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="C.O." sheetId="2" r:id="rId1"/>
     <sheet name="C.O. 3" sheetId="3" r:id="rId2"/>
-    <sheet name="76A00424M" sheetId="15" r:id="rId3"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -38,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="222" uniqueCount="88">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="177" uniqueCount="59">
   <si>
     <t xml:space="preserve">DESCRIPTION OF GOOD (S) </t>
   </si>
@@ -190,85 +189,6 @@
     <t>obed.erives@leonicables.com</t>
   </si>
   <si>
-    <t>DESCRIPTION OF PRODUCT TO EXPORT</t>
-  </si>
-  <si>
-    <t>COMERCIAL VALUE OF GOODS</t>
-  </si>
-  <si>
-    <t>DESCRIPTION ON INVOICE/PART#</t>
-  </si>
-  <si>
-    <t>UNIT MEASURE</t>
-  </si>
-  <si>
-    <t>CUSTOM TARIFF</t>
-  </si>
-  <si>
-    <t>CUSTOMER NUMBER)</t>
-  </si>
-  <si>
-    <t>MARKUP</t>
-  </si>
-  <si>
-    <t>F.O.B USD VALUE</t>
-  </si>
-  <si>
-    <t>KM</t>
-  </si>
-  <si>
-    <t>8544499904</t>
-  </si>
-  <si>
-    <t/>
-  </si>
-  <si>
-    <t>BREAKDOWN OF THE ORIGINATING SUPPLIES USED IN THE MANUFACTURE OF THE MERCHANDISE</t>
-  </si>
-  <si>
-    <t>Name of the original supplies (raw materials, parts and pieces)</t>
-  </si>
-  <si>
-    <t>QTY/KG</t>
-  </si>
-  <si>
-    <t>PU/KG</t>
-  </si>
-  <si>
-    <t>VALUE IN USD</t>
-  </si>
-  <si>
-    <t>MEXICO</t>
-  </si>
-  <si>
-    <t>USA</t>
-  </si>
-  <si>
-    <t>SUM OF ORIGINATING SUPPLIES</t>
-  </si>
-  <si>
-    <t>BREAKDOWN OF NON-ORIGINATING SUPPLIES USED IN THE MANUFACTURE OF THE GOODS</t>
-  </si>
-  <si>
-    <t>ALEMANIA</t>
-  </si>
-  <si>
-    <t>Regional Content Index</t>
-  </si>
-  <si>
-    <t>ICR= (Sum of originating supplies+markup)*100
-  Comercial value of goods FOB</t>
-  </si>
-  <si>
-    <t>ICR=</t>
-  </si>
-  <si>
-    <t>*100</t>
-  </si>
-  <si>
-    <t>Nombre y Firma del Representante Legal:__________________________________</t>
-  </si>
-  <si>
     <t>8544.49</t>
   </si>
   <si>
@@ -291,15 +211,6 @@
   </si>
   <si>
     <t xml:space="preserve">Customer Part Number </t>
-  </si>
-  <si>
-    <t xml:space="preserve">Customer Part Number / Customer Name </t>
-  </si>
-  <si>
-    <t xml:space="preserve">Leoni Part Number // leoni Part Name </t>
-  </si>
-  <si>
-    <t>Component Number / Component Name</t>
   </si>
   <si>
     <t>SEE ATTACHED</t>
@@ -309,13 +220,11 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="4">
+  <numFmts count="2">
     <numFmt numFmtId="164" formatCode="m/d/yy;@"/>
     <numFmt numFmtId="165" formatCode="mm/dd/yy;@"/>
-    <numFmt numFmtId="166" formatCode="0.000"/>
-    <numFmt numFmtId="167" formatCode="0.000%"/>
   </numFmts>
-  <fonts count="31">
+  <fonts count="21">
     <font>
       <sz val="10"/>
       <name val="Arial"/>
@@ -426,67 +335,6 @@
       <family val="2"/>
     </font>
     <font>
-      <b/>
-      <sz val="22"/>
-      <name val="Arial"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="7"/>
-      <color indexed="9"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="7"/>
-      <color indexed="9"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="7"/>
-      <color indexed="8"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="7"/>
-      <color indexed="8"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-    </font>
-    <font>
       <sz val="8"/>
       <color indexed="8"/>
       <name val="Arial"/>
@@ -499,7 +347,7 @@
       <family val="2"/>
     </font>
   </fonts>
-  <fills count="7">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -518,23 +366,8 @@
         <bgColor indexed="22"/>
       </patternFill>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor indexed="18"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor indexed="41"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor indexed="22"/>
-      </patternFill>
-    </fill>
   </fills>
-  <borders count="20">
+  <borders count="19">
     <border>
       <left/>
       <right/>
@@ -740,28 +573,13 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="16" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="17" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="182">
+  <cellXfs count="168">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="6" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
@@ -949,27 +767,6 @@
     <xf numFmtId="0" fontId="15" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="22" fillId="4" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="5" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="6" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="166" fontId="25" fillId="0" borderId="19" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="166" fontId="26" fillId="0" borderId="19" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="166" fontId="27" fillId="0" borderId="19" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="167" fontId="28" fillId="0" borderId="19" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1"/>
@@ -992,7 +789,7 @@
     <xf numFmtId="0" fontId="5" fillId="2" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="29" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="19" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="2" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1010,182 +807,163 @@
     <xf numFmtId="0" fontId="5" fillId="2" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="8" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="5" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="5" fillId="2" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="20" fillId="2" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="20" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="20" fillId="2" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="20" fillId="2" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="20" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="20" fillId="2" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="3" fillId="2" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="3" fillId="2" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="3" fillId="2" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="2" fillId="2" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="2" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="2" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="2" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="0" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="2" fontId="5" fillId="2" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="5" fillId="2" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="15" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="15" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="15" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="2" fontId="5" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="5" fillId="2" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="5" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="2" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="4" fillId="2" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="0" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="2" fontId="5" fillId="2" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="5" fillId="2" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="14" fontId="3" fillId="2" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="3" fillId="2" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="3" fillId="2" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="2" fillId="2" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="14" fontId="2" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="8" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="29" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="29" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="166" fontId="25" fillId="0" borderId="19" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="5" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="6" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="166" fontId="20" fillId="0" borderId="19" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="4" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="30" fillId="2" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="30" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="30" fillId="2" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="30" fillId="2" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="30" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="30" fillId="2" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -1954,30 +1732,30 @@
       </c>
     </row>
     <row r="2" spans="2:10" ht="14">
-      <c r="B2" s="129" t="s">
+      <c r="B2" s="149" t="s">
         <v>20</v>
       </c>
-      <c r="C2" s="130"/>
-      <c r="D2" s="130"/>
-      <c r="E2" s="130"/>
-      <c r="F2" s="130"/>
-      <c r="G2" s="130"/>
-      <c r="H2" s="130"/>
-      <c r="I2" s="130"/>
-      <c r="J2" s="131"/>
+      <c r="C2" s="150"/>
+      <c r="D2" s="150"/>
+      <c r="E2" s="150"/>
+      <c r="F2" s="150"/>
+      <c r="G2" s="150"/>
+      <c r="H2" s="150"/>
+      <c r="I2" s="150"/>
+      <c r="J2" s="151"/>
     </row>
     <row r="3" spans="2:10" ht="27" customHeight="1">
-      <c r="B3" s="132" t="s">
+      <c r="B3" s="152" t="s">
         <v>21</v>
       </c>
-      <c r="C3" s="133"/>
-      <c r="D3" s="133"/>
-      <c r="E3" s="133"/>
-      <c r="F3" s="133"/>
-      <c r="G3" s="133"/>
-      <c r="H3" s="133"/>
-      <c r="I3" s="133"/>
-      <c r="J3" s="134"/>
+      <c r="C3" s="153"/>
+      <c r="D3" s="153"/>
+      <c r="E3" s="153"/>
+      <c r="F3" s="153"/>
+      <c r="G3" s="153"/>
+      <c r="H3" s="153"/>
+      <c r="I3" s="153"/>
+      <c r="J3" s="154"/>
     </row>
     <row r="4" spans="2:10" ht="8.25" customHeight="1" thickBot="1">
       <c r="B4" s="10"/>
@@ -2166,7 +1944,7 @@
       <c r="C16" s="6"/>
       <c r="D16" s="1"/>
       <c r="E16" s="22" t="s">
-        <v>82</v>
+        <v>56</v>
       </c>
       <c r="G16" s="5"/>
       <c r="H16" s="5"/>
@@ -2238,10 +2016,10 @@
       <c r="D21" s="9"/>
       <c r="E21" s="9"/>
       <c r="F21" s="44"/>
-      <c r="G21" s="135" t="s">
+      <c r="G21" s="155" t="s">
         <v>2</v>
       </c>
-      <c r="H21" s="136"/>
+      <c r="H21" s="156"/>
       <c r="I21" s="47" t="s">
         <v>6</v>
       </c>
@@ -2257,10 +2035,10 @@
       <c r="D22" s="1"/>
       <c r="E22" s="1"/>
       <c r="F22" s="41"/>
-      <c r="G22" s="137" t="s">
+      <c r="G22" s="157" t="s">
         <v>3</v>
       </c>
-      <c r="H22" s="128"/>
+      <c r="H22" s="158"/>
       <c r="I22" s="37" t="s">
         <v>25</v>
       </c>
@@ -2276,10 +2054,10 @@
       <c r="D23" s="1"/>
       <c r="E23" s="1"/>
       <c r="F23" s="41"/>
-      <c r="G23" s="137" t="s">
+      <c r="G23" s="157" t="s">
         <v>4</v>
       </c>
-      <c r="H23" s="128"/>
+      <c r="H23" s="158"/>
       <c r="I23" s="37" t="s">
         <v>7</v>
       </c>
@@ -2293,224 +2071,224 @@
       <c r="D24" s="1"/>
       <c r="E24" s="1"/>
       <c r="F24" s="41"/>
-      <c r="G24" s="140" t="s">
+      <c r="G24" s="159" t="s">
         <v>5</v>
       </c>
-      <c r="H24" s="141"/>
+      <c r="H24" s="160"/>
       <c r="I24" s="39"/>
       <c r="J24" s="40"/>
     </row>
     <row r="25" spans="2:10" ht="13" customHeight="1">
-      <c r="B25" s="176" t="s">
-        <v>87</v>
-      </c>
-      <c r="C25" s="177"/>
-      <c r="D25" s="177"/>
-      <c r="E25" s="177"/>
-      <c r="F25" s="178"/>
-      <c r="G25" s="135"/>
-      <c r="H25" s="144"/>
-      <c r="I25" s="114"/>
-      <c r="J25" s="115"/>
+      <c r="B25" s="126" t="s">
+        <v>58</v>
+      </c>
+      <c r="C25" s="127"/>
+      <c r="D25" s="127"/>
+      <c r="E25" s="127"/>
+      <c r="F25" s="128"/>
+      <c r="G25" s="155"/>
+      <c r="H25" s="161"/>
+      <c r="I25" s="107"/>
+      <c r="J25" s="108"/>
     </row>
     <row r="26" spans="2:10" ht="13.5" customHeight="1">
-      <c r="B26" s="179"/>
-      <c r="C26" s="180"/>
-      <c r="D26" s="180"/>
-      <c r="E26" s="180"/>
-      <c r="F26" s="181"/>
-      <c r="G26" s="138"/>
-      <c r="H26" s="139"/>
-      <c r="I26" s="116"/>
-      <c r="J26" s="117"/>
+      <c r="B26" s="129"/>
+      <c r="C26" s="130"/>
+      <c r="D26" s="130"/>
+      <c r="E26" s="130"/>
+      <c r="F26" s="131"/>
+      <c r="G26" s="147"/>
+      <c r="H26" s="148"/>
+      <c r="I26" s="109"/>
+      <c r="J26" s="110"/>
     </row>
     <row r="27" spans="2:10" ht="13" customHeight="1">
-      <c r="B27" s="179"/>
-      <c r="C27" s="180"/>
-      <c r="D27" s="180"/>
-      <c r="E27" s="180"/>
-      <c r="F27" s="181"/>
-      <c r="G27" s="138"/>
-      <c r="H27" s="139"/>
-      <c r="I27" s="116"/>
-      <c r="J27" s="117"/>
+      <c r="B27" s="129"/>
+      <c r="C27" s="130"/>
+      <c r="D27" s="130"/>
+      <c r="E27" s="130"/>
+      <c r="F27" s="131"/>
+      <c r="G27" s="147"/>
+      <c r="H27" s="148"/>
+      <c r="I27" s="109"/>
+      <c r="J27" s="110"/>
     </row>
     <row r="28" spans="2:10" ht="13" customHeight="1">
-      <c r="B28" s="179"/>
-      <c r="C28" s="180"/>
-      <c r="D28" s="180"/>
-      <c r="E28" s="180"/>
-      <c r="F28" s="181"/>
-      <c r="G28" s="167"/>
-      <c r="H28" s="168"/>
-      <c r="I28" s="118"/>
-      <c r="J28" s="119"/>
+      <c r="B28" s="129"/>
+      <c r="C28" s="130"/>
+      <c r="D28" s="130"/>
+      <c r="E28" s="130"/>
+      <c r="F28" s="131"/>
+      <c r="G28" s="119"/>
+      <c r="H28" s="120"/>
+      <c r="I28" s="111"/>
+      <c r="J28" s="112"/>
     </row>
     <row r="29" spans="2:10">
-      <c r="B29" s="147" t="s">
+      <c r="B29" s="121" t="s">
         <v>10</v>
       </c>
-      <c r="C29" s="148"/>
-      <c r="D29" s="142"/>
-      <c r="E29" s="142"/>
-      <c r="F29" s="143" t="s">
+      <c r="C29" s="123"/>
+      <c r="D29" s="124"/>
+      <c r="E29" s="124"/>
+      <c r="F29" s="125" t="s">
         <v>10</v>
       </c>
-      <c r="G29" s="167"/>
-      <c r="H29" s="168"/>
-      <c r="I29" s="118"/>
-      <c r="J29" s="119"/>
+      <c r="G29" s="119"/>
+      <c r="H29" s="120"/>
+      <c r="I29" s="111"/>
+      <c r="J29" s="112"/>
     </row>
     <row r="30" spans="2:10">
-      <c r="B30" s="147" t="s">
+      <c r="B30" s="121" t="s">
         <v>10</v>
       </c>
-      <c r="C30" s="148"/>
-      <c r="D30" s="142"/>
-      <c r="E30" s="142"/>
-      <c r="F30" s="143" t="s">
+      <c r="C30" s="123"/>
+      <c r="D30" s="124"/>
+      <c r="E30" s="124"/>
+      <c r="F30" s="125" t="s">
         <v>10</v>
       </c>
-      <c r="G30" s="167"/>
-      <c r="H30" s="168"/>
-      <c r="I30" s="118"/>
-      <c r="J30" s="119"/>
+      <c r="G30" s="119"/>
+      <c r="H30" s="120"/>
+      <c r="I30" s="111"/>
+      <c r="J30" s="112"/>
     </row>
     <row r="31" spans="2:10">
-      <c r="B31" s="147" t="s">
+      <c r="B31" s="121" t="s">
         <v>10</v>
       </c>
-      <c r="C31" s="148"/>
-      <c r="D31" s="142"/>
-      <c r="E31" s="142"/>
-      <c r="F31" s="143" t="s">
+      <c r="C31" s="123"/>
+      <c r="D31" s="124"/>
+      <c r="E31" s="124"/>
+      <c r="F31" s="125" t="s">
         <v>10</v>
       </c>
-      <c r="G31" s="167"/>
-      <c r="H31" s="168"/>
-      <c r="I31" s="118"/>
-      <c r="J31" s="119"/>
+      <c r="G31" s="119"/>
+      <c r="H31" s="120"/>
+      <c r="I31" s="111"/>
+      <c r="J31" s="112"/>
     </row>
     <row r="32" spans="2:10">
-      <c r="B32" s="147" t="s">
+      <c r="B32" s="121" t="s">
         <v>10</v>
       </c>
-      <c r="C32" s="148"/>
-      <c r="D32" s="142"/>
-      <c r="E32" s="142"/>
-      <c r="F32" s="143" t="s">
+      <c r="C32" s="123"/>
+      <c r="D32" s="124"/>
+      <c r="E32" s="124"/>
+      <c r="F32" s="125" t="s">
         <v>10</v>
       </c>
-      <c r="G32" s="147"/>
-      <c r="H32" s="161"/>
-      <c r="I32" s="118"/>
-      <c r="J32" s="119"/>
+      <c r="G32" s="121"/>
+      <c r="H32" s="122"/>
+      <c r="I32" s="111"/>
+      <c r="J32" s="112"/>
     </row>
     <row r="33" spans="2:10">
-      <c r="B33" s="147" t="s">
+      <c r="B33" s="121" t="s">
         <v>10</v>
       </c>
-      <c r="C33" s="148"/>
-      <c r="D33" s="142"/>
-      <c r="E33" s="142"/>
-      <c r="F33" s="143" t="s">
+      <c r="C33" s="123"/>
+      <c r="D33" s="124"/>
+      <c r="E33" s="124"/>
+      <c r="F33" s="125" t="s">
         <v>10</v>
       </c>
-      <c r="G33" s="147"/>
-      <c r="H33" s="161"/>
-      <c r="I33" s="118"/>
-      <c r="J33" s="119"/>
+      <c r="G33" s="121"/>
+      <c r="H33" s="122"/>
+      <c r="I33" s="111"/>
+      <c r="J33" s="112"/>
     </row>
     <row r="34" spans="2:10">
-      <c r="B34" s="147" t="s">
+      <c r="B34" s="121" t="s">
         <v>10</v>
       </c>
-      <c r="C34" s="148"/>
-      <c r="D34" s="142"/>
-      <c r="E34" s="142"/>
-      <c r="F34" s="143" t="s">
+      <c r="C34" s="123"/>
+      <c r="D34" s="124"/>
+      <c r="E34" s="124"/>
+      <c r="F34" s="125" t="s">
         <v>10</v>
       </c>
-      <c r="G34" s="147"/>
-      <c r="H34" s="161"/>
-      <c r="I34" s="118"/>
-      <c r="J34" s="119"/>
+      <c r="G34" s="121"/>
+      <c r="H34" s="122"/>
+      <c r="I34" s="111"/>
+      <c r="J34" s="112"/>
     </row>
     <row r="35" spans="2:10">
-      <c r="B35" s="147" t="s">
+      <c r="B35" s="121" t="s">
         <v>10</v>
       </c>
-      <c r="C35" s="148"/>
-      <c r="D35" s="142"/>
-      <c r="E35" s="142"/>
-      <c r="F35" s="143"/>
-      <c r="G35" s="147"/>
-      <c r="H35" s="161"/>
-      <c r="I35" s="118"/>
-      <c r="J35" s="119"/>
+      <c r="C35" s="123"/>
+      <c r="D35" s="124"/>
+      <c r="E35" s="124"/>
+      <c r="F35" s="125"/>
+      <c r="G35" s="121"/>
+      <c r="H35" s="122"/>
+      <c r="I35" s="111"/>
+      <c r="J35" s="112"/>
     </row>
     <row r="36" spans="2:10">
-      <c r="B36" s="147" t="s">
+      <c r="B36" s="121" t="s">
         <v>10</v>
       </c>
-      <c r="C36" s="148"/>
-      <c r="D36" s="142"/>
-      <c r="E36" s="142"/>
-      <c r="F36" s="143"/>
-      <c r="G36" s="147"/>
-      <c r="H36" s="161"/>
-      <c r="I36" s="118"/>
-      <c r="J36" s="119"/>
+      <c r="C36" s="123"/>
+      <c r="D36" s="124"/>
+      <c r="E36" s="124"/>
+      <c r="F36" s="125"/>
+      <c r="G36" s="121"/>
+      <c r="H36" s="122"/>
+      <c r="I36" s="111"/>
+      <c r="J36" s="112"/>
     </row>
     <row r="37" spans="2:10">
-      <c r="B37" s="147"/>
-      <c r="C37" s="148"/>
-      <c r="D37" s="142"/>
-      <c r="E37" s="142"/>
-      <c r="F37" s="143"/>
-      <c r="G37" s="147"/>
-      <c r="H37" s="161"/>
-      <c r="I37" s="118"/>
-      <c r="J37" s="119"/>
+      <c r="B37" s="121"/>
+      <c r="C37" s="123"/>
+      <c r="D37" s="124"/>
+      <c r="E37" s="124"/>
+      <c r="F37" s="125"/>
+      <c r="G37" s="121"/>
+      <c r="H37" s="122"/>
+      <c r="I37" s="111"/>
+      <c r="J37" s="112"/>
     </row>
     <row r="38" spans="2:10">
-      <c r="B38" s="147"/>
-      <c r="C38" s="148"/>
-      <c r="D38" s="142"/>
-      <c r="E38" s="142"/>
-      <c r="F38" s="143"/>
-      <c r="G38" s="147"/>
-      <c r="H38" s="161"/>
-      <c r="I38" s="118"/>
-      <c r="J38" s="119"/>
+      <c r="B38" s="121"/>
+      <c r="C38" s="123"/>
+      <c r="D38" s="124"/>
+      <c r="E38" s="124"/>
+      <c r="F38" s="125"/>
+      <c r="G38" s="121"/>
+      <c r="H38" s="122"/>
+      <c r="I38" s="111"/>
+      <c r="J38" s="112"/>
     </row>
     <row r="39" spans="2:10">
-      <c r="B39" s="147"/>
-      <c r="C39" s="148"/>
-      <c r="D39" s="142"/>
-      <c r="E39" s="142"/>
-      <c r="F39" s="143"/>
-      <c r="G39" s="147"/>
-      <c r="H39" s="161"/>
-      <c r="I39" s="118"/>
-      <c r="J39" s="119"/>
+      <c r="B39" s="121"/>
+      <c r="C39" s="123"/>
+      <c r="D39" s="124"/>
+      <c r="E39" s="124"/>
+      <c r="F39" s="125"/>
+      <c r="G39" s="121"/>
+      <c r="H39" s="122"/>
+      <c r="I39" s="111"/>
+      <c r="J39" s="112"/>
     </row>
     <row r="40" spans="2:10" ht="14" thickBot="1">
-      <c r="B40" s="159"/>
-      <c r="C40" s="160"/>
-      <c r="D40" s="150"/>
-      <c r="E40" s="150"/>
-      <c r="F40" s="151"/>
-      <c r="G40" s="159"/>
-      <c r="H40" s="162"/>
-      <c r="I40" s="121"/>
-      <c r="J40" s="120"/>
+      <c r="B40" s="137"/>
+      <c r="C40" s="138"/>
+      <c r="D40" s="143"/>
+      <c r="E40" s="143"/>
+      <c r="F40" s="144"/>
+      <c r="G40" s="137"/>
+      <c r="H40" s="139"/>
+      <c r="I40" s="114"/>
+      <c r="J40" s="113"/>
     </row>
     <row r="41" spans="2:10" ht="14" thickBot="1">
-      <c r="B41" s="152" t="s">
+      <c r="B41" s="145" t="s">
         <v>29</v>
       </c>
-      <c r="C41" s="153"/>
+      <c r="C41" s="146"/>
       <c r="D41" s="6" t="s">
         <v>28</v>
       </c>
@@ -2659,8 +2437,8 @@
       <c r="J52" s="12"/>
     </row>
     <row r="53" spans="2:10" ht="20.25" customHeight="1">
-      <c r="B53" s="163"/>
-      <c r="C53" s="164"/>
+      <c r="B53" s="115"/>
+      <c r="C53" s="116"/>
       <c r="D53" s="1"/>
       <c r="E53" s="83" t="str">
         <f>B6</f>
@@ -2673,8 +2451,8 @@
       <c r="J53" s="12"/>
     </row>
     <row r="54" spans="2:10" ht="13.5" customHeight="1" thickBot="1">
-      <c r="B54" s="165"/>
-      <c r="C54" s="166"/>
+      <c r="B54" s="117"/>
+      <c r="C54" s="118"/>
       <c r="D54" s="1"/>
       <c r="E54" s="25"/>
       <c r="F54" s="62"/>
@@ -2684,8 +2462,8 @@
       <c r="J54" s="12"/>
     </row>
     <row r="55" spans="2:10" ht="9.75" customHeight="1">
-      <c r="B55" s="147"/>
-      <c r="C55" s="148"/>
+      <c r="B55" s="121"/>
+      <c r="C55" s="123"/>
       <c r="D55" s="1"/>
       <c r="E55" s="1"/>
       <c r="F55" s="5"/>
@@ -2703,15 +2481,15 @@
       <c r="E56" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="F56" s="149"/>
-      <c r="G56" s="149"/>
+      <c r="F56" s="142"/>
+      <c r="G56" s="142"/>
       <c r="H56" s="56"/>
       <c r="I56" s="1"/>
       <c r="J56" s="12"/>
     </row>
     <row r="57" spans="2:10" ht="7.5" customHeight="1" thickBot="1">
-      <c r="B57" s="157"/>
-      <c r="C57" s="158"/>
+      <c r="B57" s="135"/>
+      <c r="C57" s="136"/>
       <c r="D57" s="57"/>
       <c r="E57" s="58"/>
       <c r="F57" s="59"/>
@@ -2726,13 +2504,13 @@
       </c>
       <c r="C58" s="65"/>
       <c r="D58" s="42"/>
-      <c r="E58" s="154" t="s">
+      <c r="E58" s="132" t="s">
         <v>46</v>
       </c>
-      <c r="F58" s="155"/>
-      <c r="G58" s="155"/>
-      <c r="H58" s="155"/>
-      <c r="I58" s="156"/>
+      <c r="F58" s="133"/>
+      <c r="G58" s="133"/>
+      <c r="H58" s="133"/>
+      <c r="I58" s="134"/>
       <c r="J58" s="12"/>
     </row>
     <row r="59" spans="2:10" ht="12.75" customHeight="1">
@@ -2756,11 +2534,11 @@
       <c r="J60" s="48"/>
     </row>
     <row r="61" spans="2:10" ht="14" thickBot="1">
-      <c r="B61" s="145">
+      <c r="B61" s="140">
         <f ca="1">TODAY()</f>
-        <v>46092</v>
-      </c>
-      <c r="C61" s="146"/>
+        <v>46105</v>
+      </c>
+      <c r="C61" s="141"/>
       <c r="E61" s="66" t="s">
         <v>42</v>
       </c>
@@ -2787,19 +2565,29 @@
     </row>
   </sheetData>
   <mergeCells count="54">
-    <mergeCell ref="B53:C54"/>
-    <mergeCell ref="G28:H28"/>
-    <mergeCell ref="G29:H29"/>
-    <mergeCell ref="G30:H30"/>
-    <mergeCell ref="G31:H31"/>
-    <mergeCell ref="G32:H32"/>
-    <mergeCell ref="G36:H36"/>
-    <mergeCell ref="G37:H37"/>
-    <mergeCell ref="B30:C30"/>
-    <mergeCell ref="D30:F30"/>
-    <mergeCell ref="B34:C34"/>
-    <mergeCell ref="D34:F34"/>
-    <mergeCell ref="B25:F28"/>
+    <mergeCell ref="G24:H24"/>
+    <mergeCell ref="G25:H25"/>
+    <mergeCell ref="B2:J2"/>
+    <mergeCell ref="B3:J3"/>
+    <mergeCell ref="G21:H21"/>
+    <mergeCell ref="G22:H22"/>
+    <mergeCell ref="G23:H23"/>
+    <mergeCell ref="B61:C61"/>
+    <mergeCell ref="B35:C35"/>
+    <mergeCell ref="D35:F35"/>
+    <mergeCell ref="B32:C32"/>
+    <mergeCell ref="D32:F32"/>
+    <mergeCell ref="F56:G56"/>
+    <mergeCell ref="B38:C38"/>
+    <mergeCell ref="D38:F38"/>
+    <mergeCell ref="B39:C39"/>
+    <mergeCell ref="D39:F39"/>
+    <mergeCell ref="D40:F40"/>
+    <mergeCell ref="B36:C36"/>
+    <mergeCell ref="D36:F36"/>
+    <mergeCell ref="B41:C41"/>
+    <mergeCell ref="B55:C55"/>
+    <mergeCell ref="B37:C37"/>
     <mergeCell ref="E58:I58"/>
     <mergeCell ref="B29:C29"/>
     <mergeCell ref="D29:F29"/>
@@ -2816,31 +2604,21 @@
     <mergeCell ref="G33:H33"/>
     <mergeCell ref="G34:H34"/>
     <mergeCell ref="G35:H35"/>
-    <mergeCell ref="B61:C61"/>
-    <mergeCell ref="B35:C35"/>
-    <mergeCell ref="D35:F35"/>
-    <mergeCell ref="B32:C32"/>
-    <mergeCell ref="D32:F32"/>
-    <mergeCell ref="F56:G56"/>
-    <mergeCell ref="B38:C38"/>
-    <mergeCell ref="D38:F38"/>
-    <mergeCell ref="B39:C39"/>
-    <mergeCell ref="D39:F39"/>
-    <mergeCell ref="D40:F40"/>
-    <mergeCell ref="B36:C36"/>
-    <mergeCell ref="D36:F36"/>
-    <mergeCell ref="B41:C41"/>
-    <mergeCell ref="B55:C55"/>
-    <mergeCell ref="B37:C37"/>
+    <mergeCell ref="B53:C54"/>
+    <mergeCell ref="G28:H28"/>
+    <mergeCell ref="G29:H29"/>
+    <mergeCell ref="G30:H30"/>
+    <mergeCell ref="G31:H31"/>
+    <mergeCell ref="G32:H32"/>
+    <mergeCell ref="G36:H36"/>
+    <mergeCell ref="G37:H37"/>
+    <mergeCell ref="B30:C30"/>
+    <mergeCell ref="D30:F30"/>
+    <mergeCell ref="B34:C34"/>
+    <mergeCell ref="D34:F34"/>
+    <mergeCell ref="B25:F28"/>
     <mergeCell ref="G26:H26"/>
     <mergeCell ref="G27:H27"/>
-    <mergeCell ref="B2:J2"/>
-    <mergeCell ref="B3:J3"/>
-    <mergeCell ref="G21:H21"/>
-    <mergeCell ref="G22:H22"/>
-    <mergeCell ref="G23:H23"/>
-    <mergeCell ref="G24:H24"/>
-    <mergeCell ref="G25:H25"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink ref="C12" r:id="rId1" xr:uid="{00000000-0004-0000-0000-000000000000}"/>
@@ -2881,28 +2659,28 @@
       </c>
     </row>
     <row r="2" spans="2:9" ht="14">
-      <c r="B2" s="129" t="s">
+      <c r="B2" s="149" t="s">
         <v>20</v>
       </c>
-      <c r="C2" s="130"/>
-      <c r="D2" s="130"/>
-      <c r="E2" s="130"/>
-      <c r="F2" s="130"/>
-      <c r="G2" s="130"/>
-      <c r="H2" s="130"/>
-      <c r="I2" s="131"/>
+      <c r="C2" s="150"/>
+      <c r="D2" s="150"/>
+      <c r="E2" s="150"/>
+      <c r="F2" s="150"/>
+      <c r="G2" s="150"/>
+      <c r="H2" s="150"/>
+      <c r="I2" s="151"/>
     </row>
     <row r="3" spans="2:9" ht="27" customHeight="1">
-      <c r="B3" s="132" t="s">
+      <c r="B3" s="152" t="s">
         <v>21</v>
       </c>
-      <c r="C3" s="133"/>
-      <c r="D3" s="133"/>
-      <c r="E3" s="133"/>
-      <c r="F3" s="133"/>
-      <c r="G3" s="133"/>
-      <c r="H3" s="133"/>
-      <c r="I3" s="134"/>
+      <c r="C3" s="153"/>
+      <c r="D3" s="153"/>
+      <c r="E3" s="153"/>
+      <c r="F3" s="153"/>
+      <c r="G3" s="153"/>
+      <c r="H3" s="153"/>
+      <c r="I3" s="154"/>
     </row>
     <row r="4" spans="2:9" ht="8.25" customHeight="1" thickBot="1">
       <c r="B4" s="10"/>
@@ -2919,10 +2697,10 @@
       <c r="C5" s="28"/>
       <c r="D5" s="9"/>
       <c r="E5" s="44"/>
-      <c r="F5" s="135" t="s">
+      <c r="F5" s="155" t="s">
         <v>2</v>
       </c>
-      <c r="G5" s="136"/>
+      <c r="G5" s="156"/>
       <c r="H5" s="47" t="s">
         <v>6</v>
       </c>
@@ -2937,10 +2715,10 @@
       </c>
       <c r="D6" s="1"/>
       <c r="E6" s="41"/>
-      <c r="F6" s="137" t="s">
+      <c r="F6" s="157" t="s">
         <v>3</v>
       </c>
-      <c r="G6" s="128"/>
+      <c r="G6" s="158"/>
       <c r="H6" s="37" t="s">
         <v>25</v>
       </c>
@@ -2955,10 +2733,10 @@
       </c>
       <c r="D7" s="1"/>
       <c r="E7" s="41"/>
-      <c r="F7" s="137" t="s">
+      <c r="F7" s="157" t="s">
         <v>4</v>
       </c>
-      <c r="G7" s="128"/>
+      <c r="G7" s="158"/>
       <c r="H7" s="37" t="s">
         <v>7</v>
       </c>
@@ -2970,305 +2748,305 @@
       <c r="B8" s="88" t="s">
         <v>43</v>
       </c>
-      <c r="C8" s="104" t="s">
-        <v>83</v>
+      <c r="C8" s="97" t="s">
+        <v>57</v>
       </c>
       <c r="D8" s="89" t="s">
-        <v>79</v>
-      </c>
-      <c r="E8" s="104" t="s">
-        <v>80</v>
-      </c>
-      <c r="F8" s="128" t="s">
+        <v>53</v>
+      </c>
+      <c r="E8" s="97" t="s">
+        <v>54</v>
+      </c>
+      <c r="F8" s="158" t="s">
         <v>5</v>
       </c>
-      <c r="G8" s="128"/>
+      <c r="G8" s="158"/>
       <c r="H8" s="87"/>
       <c r="I8" s="38"/>
     </row>
     <row r="9" spans="2:9">
-      <c r="B9" s="107" t="s">
+      <c r="B9" s="100" t="s">
         <v>41</v>
       </c>
-      <c r="C9" s="110" t="s">
-        <v>81</v>
-      </c>
-      <c r="D9" s="108" t="s">
-        <v>81</v>
-      </c>
-      <c r="E9" s="110" t="s">
-        <v>81</v>
-      </c>
-      <c r="F9" s="126" t="s">
-        <v>76</v>
-      </c>
-      <c r="G9" s="127"/>
-      <c r="H9" s="109" t="s">
-        <v>77</v>
-      </c>
-      <c r="I9" s="107" t="s">
-        <v>78</v>
+      <c r="C9" s="103" t="s">
+        <v>55</v>
+      </c>
+      <c r="D9" s="101" t="s">
+        <v>55</v>
+      </c>
+      <c r="E9" s="103" t="s">
+        <v>55</v>
+      </c>
+      <c r="F9" s="162" t="s">
+        <v>50</v>
+      </c>
+      <c r="G9" s="163"/>
+      <c r="H9" s="102" t="s">
+        <v>51</v>
+      </c>
+      <c r="I9" s="100" t="s">
+        <v>52</v>
       </c>
     </row>
     <row r="10" spans="2:9">
-      <c r="B10" s="105" t="s">
+      <c r="B10" s="98" t="s">
         <v>41</v>
       </c>
       <c r="C10" s="55" t="s">
-        <v>81</v>
-      </c>
-      <c r="D10" s="112" t="s">
-        <v>81</v>
+        <v>55</v>
+      </c>
+      <c r="D10" s="105" t="s">
+        <v>55</v>
       </c>
       <c r="E10" s="55" t="s">
-        <v>81</v>
-      </c>
-      <c r="F10" s="124" t="s">
-        <v>76</v>
-      </c>
-      <c r="G10" s="125"/>
+        <v>55</v>
+      </c>
+      <c r="F10" s="164" t="s">
+        <v>50</v>
+      </c>
+      <c r="G10" s="165"/>
       <c r="H10" t="s">
-        <v>77</v>
-      </c>
-      <c r="I10" s="105" t="s">
-        <v>78</v>
+        <v>51</v>
+      </c>
+      <c r="I10" s="98" t="s">
+        <v>52</v>
       </c>
     </row>
     <row r="11" spans="2:9">
-      <c r="B11" s="105" t="s">
+      <c r="B11" s="98" t="s">
         <v>41</v>
       </c>
       <c r="C11" s="55" t="s">
-        <v>81</v>
-      </c>
-      <c r="D11" s="112" t="s">
-        <v>81</v>
+        <v>55</v>
+      </c>
+      <c r="D11" s="105" t="s">
+        <v>55</v>
       </c>
       <c r="E11" s="55" t="s">
-        <v>81</v>
-      </c>
-      <c r="F11" s="124" t="s">
-        <v>76</v>
-      </c>
-      <c r="G11" s="125"/>
+        <v>55</v>
+      </c>
+      <c r="F11" s="164" t="s">
+        <v>50</v>
+      </c>
+      <c r="G11" s="165"/>
       <c r="H11" t="s">
-        <v>77</v>
-      </c>
-      <c r="I11" s="105" t="s">
-        <v>78</v>
+        <v>51</v>
+      </c>
+      <c r="I11" s="98" t="s">
+        <v>52</v>
       </c>
     </row>
     <row r="12" spans="2:9">
-      <c r="B12" s="105" t="s">
+      <c r="B12" s="98" t="s">
         <v>41</v>
       </c>
       <c r="C12" s="55" t="s">
-        <v>81</v>
-      </c>
-      <c r="D12" s="112" t="s">
-        <v>81</v>
+        <v>55</v>
+      </c>
+      <c r="D12" s="105" t="s">
+        <v>55</v>
       </c>
       <c r="E12" s="55" t="s">
-        <v>81</v>
-      </c>
-      <c r="F12" s="124" t="s">
-        <v>76</v>
-      </c>
-      <c r="G12" s="125"/>
+        <v>55</v>
+      </c>
+      <c r="F12" s="164" t="s">
+        <v>50</v>
+      </c>
+      <c r="G12" s="165"/>
       <c r="H12" t="s">
-        <v>77</v>
-      </c>
-      <c r="I12" s="105" t="s">
-        <v>78</v>
+        <v>51</v>
+      </c>
+      <c r="I12" s="98" t="s">
+        <v>52</v>
       </c>
     </row>
     <row r="13" spans="2:9">
-      <c r="B13" s="105" t="s">
+      <c r="B13" s="98" t="s">
         <v>41</v>
       </c>
       <c r="C13" s="55" t="s">
-        <v>81</v>
-      </c>
-      <c r="D13" s="112" t="s">
-        <v>81</v>
+        <v>55</v>
+      </c>
+      <c r="D13" s="105" t="s">
+        <v>55</v>
       </c>
       <c r="E13" s="55" t="s">
-        <v>81</v>
-      </c>
-      <c r="F13" s="124" t="s">
-        <v>76</v>
-      </c>
-      <c r="G13" s="125"/>
+        <v>55</v>
+      </c>
+      <c r="F13" s="164" t="s">
+        <v>50</v>
+      </c>
+      <c r="G13" s="165"/>
       <c r="H13" t="s">
-        <v>77</v>
-      </c>
-      <c r="I13" s="105" t="s">
-        <v>78</v>
+        <v>51</v>
+      </c>
+      <c r="I13" s="98" t="s">
+        <v>52</v>
       </c>
     </row>
     <row r="14" spans="2:9">
-      <c r="B14" s="105" t="s">
+      <c r="B14" s="98" t="s">
         <v>41</v>
       </c>
       <c r="C14" s="55" t="s">
-        <v>81</v>
-      </c>
-      <c r="D14" s="112" t="s">
-        <v>81</v>
+        <v>55</v>
+      </c>
+      <c r="D14" s="105" t="s">
+        <v>55</v>
       </c>
       <c r="E14" s="55" t="s">
-        <v>81</v>
-      </c>
-      <c r="F14" s="124" t="s">
-        <v>76</v>
-      </c>
-      <c r="G14" s="125"/>
+        <v>55</v>
+      </c>
+      <c r="F14" s="164" t="s">
+        <v>50</v>
+      </c>
+      <c r="G14" s="165"/>
       <c r="H14" t="s">
-        <v>77</v>
-      </c>
-      <c r="I14" s="105" t="s">
-        <v>78</v>
+        <v>51</v>
+      </c>
+      <c r="I14" s="98" t="s">
+        <v>52</v>
       </c>
     </row>
     <row r="15" spans="2:9">
-      <c r="B15" s="105" t="s">
+      <c r="B15" s="98" t="s">
         <v>41</v>
       </c>
       <c r="C15" s="55" t="s">
-        <v>81</v>
-      </c>
-      <c r="D15" s="112" t="s">
-        <v>81</v>
+        <v>55</v>
+      </c>
+      <c r="D15" s="105" t="s">
+        <v>55</v>
       </c>
       <c r="E15" s="55" t="s">
-        <v>81</v>
-      </c>
-      <c r="F15" s="124" t="s">
-        <v>76</v>
-      </c>
-      <c r="G15" s="125"/>
+        <v>55</v>
+      </c>
+      <c r="F15" s="164" t="s">
+        <v>50</v>
+      </c>
+      <c r="G15" s="165"/>
       <c r="H15" t="s">
-        <v>77</v>
-      </c>
-      <c r="I15" s="105" t="s">
-        <v>78</v>
+        <v>51</v>
+      </c>
+      <c r="I15" s="98" t="s">
+        <v>52</v>
       </c>
     </row>
     <row r="16" spans="2:9">
-      <c r="B16" s="105" t="s">
+      <c r="B16" s="98" t="s">
         <v>41</v>
       </c>
       <c r="C16" s="55" t="s">
-        <v>81</v>
-      </c>
-      <c r="D16" s="112" t="s">
-        <v>81</v>
+        <v>55</v>
+      </c>
+      <c r="D16" s="105" t="s">
+        <v>55</v>
       </c>
       <c r="E16" s="55" t="s">
-        <v>81</v>
-      </c>
-      <c r="F16" s="124" t="s">
-        <v>76</v>
-      </c>
-      <c r="G16" s="125"/>
+        <v>55</v>
+      </c>
+      <c r="F16" s="164" t="s">
+        <v>50</v>
+      </c>
+      <c r="G16" s="165"/>
       <c r="H16" t="s">
-        <v>77</v>
-      </c>
-      <c r="I16" s="105" t="s">
-        <v>78</v>
+        <v>51</v>
+      </c>
+      <c r="I16" s="98" t="s">
+        <v>52</v>
       </c>
     </row>
     <row r="17" spans="2:9">
-      <c r="B17" s="105" t="s">
+      <c r="B17" s="98" t="s">
         <v>41</v>
       </c>
       <c r="C17" s="55" t="s">
-        <v>81</v>
-      </c>
-      <c r="D17" s="112" t="s">
-        <v>81</v>
+        <v>55</v>
+      </c>
+      <c r="D17" s="105" t="s">
+        <v>55</v>
       </c>
       <c r="E17" s="55" t="s">
-        <v>81</v>
-      </c>
-      <c r="F17" s="124" t="s">
-        <v>76</v>
-      </c>
-      <c r="G17" s="125"/>
+        <v>55</v>
+      </c>
+      <c r="F17" s="164" t="s">
+        <v>50</v>
+      </c>
+      <c r="G17" s="165"/>
       <c r="H17" t="s">
-        <v>77</v>
-      </c>
-      <c r="I17" s="105" t="s">
-        <v>78</v>
+        <v>51</v>
+      </c>
+      <c r="I17" s="98" t="s">
+        <v>52</v>
       </c>
     </row>
     <row r="18" spans="2:9">
-      <c r="B18" s="105" t="s">
+      <c r="B18" s="98" t="s">
         <v>41</v>
       </c>
       <c r="C18" s="55" t="s">
-        <v>81</v>
-      </c>
-      <c r="D18" s="112" t="s">
-        <v>81</v>
+        <v>55</v>
+      </c>
+      <c r="D18" s="105" t="s">
+        <v>55</v>
       </c>
       <c r="E18" s="55" t="s">
-        <v>81</v>
-      </c>
-      <c r="F18" s="124" t="s">
-        <v>76</v>
-      </c>
-      <c r="G18" s="125"/>
+        <v>55</v>
+      </c>
+      <c r="F18" s="164" t="s">
+        <v>50</v>
+      </c>
+      <c r="G18" s="165"/>
       <c r="H18" t="s">
-        <v>77</v>
-      </c>
-      <c r="I18" s="105" t="s">
-        <v>78</v>
+        <v>51</v>
+      </c>
+      <c r="I18" s="98" t="s">
+        <v>52</v>
       </c>
     </row>
     <row r="19" spans="2:9" ht="14" thickBot="1">
-      <c r="B19" s="106" t="s">
+      <c r="B19" s="99" t="s">
         <v>41</v>
       </c>
-      <c r="C19" s="111" t="s">
-        <v>81</v>
-      </c>
-      <c r="D19" s="113" t="s">
-        <v>81</v>
-      </c>
-      <c r="E19" s="111" t="s">
-        <v>81</v>
-      </c>
-      <c r="F19" s="122" t="s">
-        <v>76</v>
-      </c>
-      <c r="G19" s="123"/>
+      <c r="C19" s="104" t="s">
+        <v>55</v>
+      </c>
+      <c r="D19" s="106" t="s">
+        <v>55</v>
+      </c>
+      <c r="E19" s="104" t="s">
+        <v>55</v>
+      </c>
+      <c r="F19" s="166" t="s">
+        <v>50</v>
+      </c>
+      <c r="G19" s="167"/>
       <c r="H19" s="68" t="s">
-        <v>77</v>
-      </c>
-      <c r="I19" s="106" t="s">
-        <v>78</v>
+        <v>51</v>
+      </c>
+      <c r="I19" s="99" t="s">
+        <v>52</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="17">
+    <mergeCell ref="F19:G19"/>
+    <mergeCell ref="F14:G14"/>
+    <mergeCell ref="F15:G15"/>
+    <mergeCell ref="F16:G16"/>
+    <mergeCell ref="F17:G17"/>
+    <mergeCell ref="F18:G18"/>
+    <mergeCell ref="F9:G9"/>
+    <mergeCell ref="F10:G10"/>
+    <mergeCell ref="F11:G11"/>
+    <mergeCell ref="F12:G12"/>
+    <mergeCell ref="F13:G13"/>
     <mergeCell ref="F8:G8"/>
     <mergeCell ref="B2:I2"/>
     <mergeCell ref="B3:I3"/>
     <mergeCell ref="F5:G5"/>
     <mergeCell ref="F6:G6"/>
     <mergeCell ref="F7:G7"/>
-    <mergeCell ref="F9:G9"/>
-    <mergeCell ref="F10:G10"/>
-    <mergeCell ref="F11:G11"/>
-    <mergeCell ref="F12:G12"/>
-    <mergeCell ref="F13:G13"/>
-    <mergeCell ref="F19:G19"/>
-    <mergeCell ref="F14:G14"/>
-    <mergeCell ref="F15:G15"/>
-    <mergeCell ref="F16:G16"/>
-    <mergeCell ref="F17:G17"/>
-    <mergeCell ref="F18:G18"/>
   </mergeCells>
   <pageMargins left="0.25" right="0.17" top="0.27" bottom="0.22" header="0.25" footer="0.2"/>
   <pageSetup scale="78" orientation="portrait" r:id="rId1"/>
@@ -3278,356 +3056,6 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0D00-000000000000}">
-  <dimension ref="B1:P31"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.5" defaultRowHeight="13"/>
-  <cols>
-    <col min="1" max="1" width="17" customWidth="1"/>
-    <col min="2" max="7" width="17.1640625" customWidth="1"/>
-    <col min="8" max="8" width="17.1640625" bestFit="1" customWidth="1"/>
-    <col min="9" max="10" width="17.1640625" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="2:12" ht="33" customHeight="1">
-      <c r="B1" s="174" t="s">
-        <v>84</v>
-      </c>
-      <c r="C1" s="172"/>
-      <c r="D1" s="172"/>
-      <c r="E1" s="172"/>
-      <c r="F1" s="172"/>
-      <c r="G1" s="172"/>
-      <c r="H1" s="172"/>
-    </row>
-    <row r="2" spans="2:12" ht="25" customHeight="1">
-      <c r="B2" s="175" t="s">
-        <v>50</v>
-      </c>
-      <c r="C2" s="172"/>
-      <c r="D2" s="172"/>
-      <c r="E2" s="172"/>
-      <c r="F2" s="172"/>
-      <c r="G2" s="172"/>
-      <c r="H2" s="97" t="s">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="3" spans="2:12" ht="45" customHeight="1">
-      <c r="B3" s="169" t="s">
-        <v>52</v>
-      </c>
-      <c r="C3" s="169"/>
-      <c r="D3" s="100" t="s">
-        <v>53</v>
-      </c>
-      <c r="E3" s="100" t="s">
-        <v>54</v>
-      </c>
-      <c r="F3" s="100" t="s">
-        <v>55</v>
-      </c>
-      <c r="G3" s="100" t="s">
-        <v>56</v>
-      </c>
-      <c r="H3" s="100" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="4" spans="2:12" ht="45" customHeight="1">
-      <c r="B4" s="173" t="s">
-        <v>85</v>
-      </c>
-      <c r="C4" s="169"/>
-      <c r="D4" s="101" t="s">
-        <v>58</v>
-      </c>
-      <c r="E4" s="101" t="s">
-        <v>59</v>
-      </c>
-      <c r="F4" s="101" t="s">
-        <v>60</v>
-      </c>
-      <c r="G4" s="101">
-        <f>H4-H13-H23</f>
-        <v>471.57097380000016</v>
-      </c>
-      <c r="H4" s="101">
-        <v>1540.3066670000001</v>
-      </c>
-    </row>
-    <row r="6" spans="2:12" ht="25" customHeight="1">
-      <c r="B6" s="170" t="s">
-        <v>61</v>
-      </c>
-      <c r="C6" s="170"/>
-      <c r="D6" s="170"/>
-      <c r="E6" s="170"/>
-      <c r="F6" s="170"/>
-      <c r="G6" s="170"/>
-      <c r="H6" s="170"/>
-    </row>
-    <row r="7" spans="2:12" ht="25" customHeight="1">
-      <c r="B7" s="170" t="s">
-        <v>62</v>
-      </c>
-      <c r="C7" s="172"/>
-      <c r="D7" s="172"/>
-      <c r="E7" s="98" t="s">
-        <v>63</v>
-      </c>
-      <c r="F7" s="98" t="s">
-        <v>64</v>
-      </c>
-      <c r="G7" s="98" t="s">
-        <v>25</v>
-      </c>
-      <c r="H7" s="98" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="8" spans="2:12" ht="22" customHeight="1">
-      <c r="B8" s="173" t="s">
-        <v>86</v>
-      </c>
-      <c r="C8" s="169"/>
-      <c r="D8" s="169"/>
-      <c r="E8" s="100">
-        <v>37.07</v>
-      </c>
-      <c r="F8" s="100">
-        <v>10.78</v>
-      </c>
-      <c r="G8" s="100" t="s">
-        <v>66</v>
-      </c>
-      <c r="H8" s="100">
-        <f>F8*E8</f>
-        <v>399.6146</v>
-      </c>
-    </row>
-    <row r="9" spans="2:12" ht="22" customHeight="1">
-      <c r="B9" s="173" t="s">
-        <v>86</v>
-      </c>
-      <c r="C9" s="169"/>
-      <c r="D9" s="169"/>
-      <c r="E9" s="100">
-        <v>37.07</v>
-      </c>
-      <c r="F9" s="100">
-        <v>11.66</v>
-      </c>
-      <c r="G9" s="100" t="s">
-        <v>67</v>
-      </c>
-      <c r="H9" s="100">
-        <f>F9*E9</f>
-        <v>432.2362</v>
-      </c>
-    </row>
-    <row r="10" spans="2:12" ht="22" customHeight="1">
-      <c r="B10" s="173" t="s">
-        <v>86</v>
-      </c>
-      <c r="C10" s="169"/>
-      <c r="D10" s="169"/>
-      <c r="E10" s="100">
-        <v>44.17</v>
-      </c>
-      <c r="F10" s="100">
-        <v>4.28</v>
-      </c>
-      <c r="G10" s="100" t="s">
-        <v>67</v>
-      </c>
-      <c r="H10" s="100">
-        <f>F10*E10</f>
-        <v>189.04760000000002</v>
-      </c>
-      <c r="L10" t="s">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="13" spans="2:12" ht="22" customHeight="1">
-      <c r="E13" s="169" t="s">
-        <v>68</v>
-      </c>
-      <c r="F13" s="169"/>
-      <c r="G13" s="169"/>
-      <c r="H13" s="100">
-        <f>SUM(H8:H12)</f>
-        <v>1020.8983999999999</v>
-      </c>
-    </row>
-    <row r="16" spans="2:12" ht="25" customHeight="1">
-      <c r="B16" s="170" t="s">
-        <v>69</v>
-      </c>
-      <c r="C16" s="170"/>
-      <c r="D16" s="170"/>
-      <c r="E16" s="170"/>
-      <c r="F16" s="170"/>
-      <c r="G16" s="170"/>
-      <c r="H16" s="170"/>
-    </row>
-    <row r="17" spans="2:16" ht="25" customHeight="1">
-      <c r="B17" s="171" t="s">
-        <v>62</v>
-      </c>
-      <c r="C17" s="172"/>
-      <c r="D17" s="172"/>
-      <c r="E17" s="99" t="s">
-        <v>63</v>
-      </c>
-      <c r="F17" s="99" t="s">
-        <v>64</v>
-      </c>
-      <c r="G17" s="99" t="s">
-        <v>25</v>
-      </c>
-      <c r="H17" s="99" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="18" spans="2:16" ht="22" customHeight="1">
-      <c r="B18" s="173" t="s">
-        <v>86</v>
-      </c>
-      <c r="C18" s="169"/>
-      <c r="D18" s="169"/>
-      <c r="E18" s="100">
-        <v>25.33</v>
-      </c>
-      <c r="F18" s="100">
-        <v>1.6308</v>
-      </c>
-      <c r="G18" s="100" t="s">
-        <v>70</v>
-      </c>
-      <c r="H18" s="100">
-        <f>F18*E18</f>
-        <v>41.308163999999998</v>
-      </c>
-      <c r="L18" t="s">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="19" spans="2:16" ht="22" customHeight="1">
-      <c r="B19" s="173" t="s">
-        <v>86</v>
-      </c>
-      <c r="C19" s="169"/>
-      <c r="D19" s="169"/>
-      <c r="E19" s="100">
-        <v>1.1000000000000001</v>
-      </c>
-      <c r="F19" s="100">
-        <v>5.9355719999999996</v>
-      </c>
-      <c r="G19" s="100" t="s">
-        <v>70</v>
-      </c>
-      <c r="H19" s="100">
-        <f>F19*E19</f>
-        <v>6.5291291999999999</v>
-      </c>
-      <c r="P19" t="s">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="23" spans="2:16" ht="22" customHeight="1">
-      <c r="E23" s="169" t="s">
-        <v>68</v>
-      </c>
-      <c r="F23" s="169"/>
-      <c r="G23" s="169"/>
-      <c r="H23" s="100">
-        <f>SUM(H18:H22)</f>
-        <v>47.837293199999998</v>
-      </c>
-    </row>
-    <row r="25" spans="2:16" ht="22" customHeight="1">
-      <c r="B25" s="169" t="s">
-        <v>71</v>
-      </c>
-      <c r="C25" s="169"/>
-      <c r="D25" s="169"/>
-    </row>
-    <row r="26" spans="2:16" ht="22" customHeight="1">
-      <c r="B26" s="169" t="s">
-        <v>72</v>
-      </c>
-      <c r="C26" s="169"/>
-      <c r="D26" s="169"/>
-    </row>
-    <row r="27" spans="2:16" ht="22" customHeight="1">
-      <c r="B27" s="169"/>
-      <c r="C27" s="169"/>
-      <c r="D27" s="169"/>
-      <c r="E27" s="102" t="s">
-        <v>73</v>
-      </c>
-      <c r="F27" s="102">
-        <f>H13+G4</f>
-        <v>1492.4693738000001</v>
-      </c>
-      <c r="G27" s="102" t="s">
-        <v>74</v>
-      </c>
-      <c r="I27" s="103">
-        <f>(F27/F28)</f>
-        <v>0.96894300711353087</v>
-      </c>
-    </row>
-    <row r="28" spans="2:16" ht="22" customHeight="1">
-      <c r="B28" s="169"/>
-      <c r="C28" s="169"/>
-      <c r="D28" s="169"/>
-      <c r="F28" s="102">
-        <f>H4</f>
-        <v>1540.3066670000001</v>
-      </c>
-    </row>
-    <row r="29" spans="2:16" ht="22" customHeight="1">
-      <c r="B29" s="169"/>
-      <c r="C29" s="169"/>
-      <c r="D29" s="169"/>
-    </row>
-    <row r="31" spans="2:16" ht="22" customHeight="1">
-      <c r="C31" s="169" t="s">
-        <v>75</v>
-      </c>
-      <c r="D31" s="169"/>
-      <c r="E31" s="169"/>
-      <c r="F31" s="169"/>
-      <c r="G31" s="169"/>
-    </row>
-  </sheetData>
-  <mergeCells count="18">
-    <mergeCell ref="B1:H1"/>
-    <mergeCell ref="B2:G2"/>
-    <mergeCell ref="B3:C3"/>
-    <mergeCell ref="B4:C4"/>
-    <mergeCell ref="B6:H6"/>
-    <mergeCell ref="B7:D7"/>
-    <mergeCell ref="B8:D8"/>
-    <mergeCell ref="B9:D9"/>
-    <mergeCell ref="B10:D10"/>
-    <mergeCell ref="E13:G13"/>
-    <mergeCell ref="B25:D25"/>
-    <mergeCell ref="B26:D29"/>
-    <mergeCell ref="C31:G31"/>
-    <mergeCell ref="B16:H16"/>
-    <mergeCell ref="B17:D17"/>
-    <mergeCell ref="B18:D18"/>
-    <mergeCell ref="B19:D19"/>
-    <mergeCell ref="E23:G23"/>
-  </mergeCells>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
 <file path=docMetadata/LabelInfo.xml><?xml version="1.0" encoding="utf-8"?>
 <clbl:labelList xmlns:clbl="http://schemas.microsoft.com/office/2020/mipLabelMetadata">
   <clbl:label id="{43c1c031-4620-46ba-8d17-94284d681a00}" enabled="1" method="Standard" siteId="{601e50db-f61c-4594-8e2e-260c58d3cfa1}" contentBits="2" removed="0"/>

</xml_diff>